<commit_message>
chore(data): batch update intraday vendas - 09:15:05
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,6 +487,117 @@
         <is>
           <t>TOTAL_VALOR_VENDA</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>147</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>70696</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H2" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>82.98</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>147</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>141361</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H3" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>147</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H4" t="n">
+        <v>789825</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>67.54000000000001</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 09:30:03
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,15 +496,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>70696</v>
+        <v>161944</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>82.98</v>
+        <v>57.06</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>141361</v>
+        <v>70696</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -549,15 +549,15 @@
         <v>46281</v>
       </c>
       <c r="H3" t="n">
-        <v>31305</v>
+        <v>33928</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>33.04</v>
+        <v>82.98</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -570,15 +570,15 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>156052</v>
+        <v>148126</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -586,17 +586,387 @@
         <v>46281</v>
       </c>
       <c r="H4" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>143529</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H5" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>72</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>140308</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H6" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>31.51</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>72</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>39233</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H7" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>147</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>141361</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>72</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>140846</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H9" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>22</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>72</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>122050</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H10" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>49.61</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>72</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>151540</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H11" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>72</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>95842</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H12" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>72</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>12521</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H13" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>147</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H14" t="n">
         <v>789825</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="J14" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 09:45:06
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,15 +496,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>161944</v>
+        <v>70696</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>57.06</v>
+        <v>82.98</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -533,15 +533,15 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>70696</v>
+        <v>98221</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -549,15 +549,15 @@
         <v>46281</v>
       </c>
       <c r="H3" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>82.98</v>
+        <v>7.35</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>148126</v>
+        <v>79510</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -586,15 +586,15 @@
         <v>46281</v>
       </c>
       <c r="H4" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>11.27</v>
+        <v>8.84</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>143529</v>
+        <v>161738</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -623,15 +623,15 @@
         <v>46281</v>
       </c>
       <c r="H5" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>21.1</v>
+        <v>16.79</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>140308</v>
+        <v>148126</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -660,15 +660,15 @@
         <v>46281</v>
       </c>
       <c r="H6" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>31.51</v>
+        <v>11.27</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>39233</v>
+        <v>143529</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>17.83</v>
+        <v>21.1</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -718,31 +718,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G8" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H8" t="n">
-        <v>31305</v>
+        <v>33928</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>33.04</v>
+        <v>31.51</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -763,7 +769,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>140846</v>
+        <v>141092</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -771,15 +777,15 @@
         <v>46281</v>
       </c>
       <c r="H9" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>22</v>
+        <v>7.29</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -800,7 +806,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>122050</v>
+        <v>154430</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -808,15 +814,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>49.61</v>
+        <v>29.46</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -837,7 +843,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>151540</v>
+        <v>39233</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -845,15 +851,15 @@
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>12.46</v>
+        <v>17.83</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -874,7 +880,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>95842</v>
+        <v>161224</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -882,15 +888,15 @@
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7.69</v>
+        <v>31.97</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -911,7 +917,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>12521</v>
+        <v>157889</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -919,15 +925,15 @@
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>12.86</v>
+        <v>8.33</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -940,15 +946,15 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>156052</v>
+        <v>144460</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -956,17 +962,380 @@
         <v>46281</v>
       </c>
       <c r="H14" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>147</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>141361</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H15" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>72</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>95842</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>46753</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H16" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>72</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>122050</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>46905</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H17" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>49.61</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>72</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>140846</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H18" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>22</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>72</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>151540</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>46569</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H19" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>72</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>152321</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H20" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>72</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>161944</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H21" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>72</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>12521</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H22" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>147</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H23" t="n">
         <v>789825</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="J23" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K23" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:00:04
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>148126</v>
+        <v>143552</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -660,15 +660,15 @@
         <v>46281</v>
       </c>
       <c r="H6" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>11.27</v>
+        <v>23.94</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>143529</v>
+        <v>157169</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -697,15 +697,15 @@
         <v>46281</v>
       </c>
       <c r="H7" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>21.1</v>
+        <v>23.7</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -726,29 +726,23 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>155062</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H8" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>31.51</v>
+        <v>63.38</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -769,7 +763,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>141092</v>
+        <v>143529</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -777,15 +771,15 @@
         <v>46281</v>
       </c>
       <c r="H9" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>7.29</v>
+        <v>21.1</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -806,7 +800,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>154430</v>
+        <v>4006</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -814,15 +808,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>29.46</v>
+        <v>12.48</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -843,23 +837,29 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>39233</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G11" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>31305</v>
+        <v>33928</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>17.83</v>
+        <v>31.51</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>161224</v>
+        <v>141092</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>31.97</v>
+        <v>7.29</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>157889</v>
+        <v>140738</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -925,15 +925,15 @@
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>8.33</v>
+        <v>29.12</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -954,23 +954,29 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>144460</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+        <v>148126</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>A90B00326</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G14" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>6.56</v>
+        <v>11.27</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -983,18 +989,24 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1007,7 +1019,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>33.04</v>
+        <v>17.83</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1028,29 +1040,23 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>154430</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H16" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>7.69</v>
+        <v>29.46</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1071,29 +1077,23 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>134701</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>49.61</v>
+        <v>9.35</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,29 +1114,23 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>140846</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2603107</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>141180</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H18" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>22</v>
+        <v>12.8</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1157,29 +1151,23 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>161224</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H19" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>12.46</v>
+        <v>31.97</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1200,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>152321</v>
+        <v>153194</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1208,15 +1196,15 @@
         <v>46281</v>
       </c>
       <c r="H20" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>8.83</v>
+        <v>55.4</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1237,29 +1225,23 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>145691</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H21" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>57.06</v>
+        <v>38.72</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1282,8 +1264,14 @@
       <c r="D22" t="n">
         <v>12521</v>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G22" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1309,15 +1297,15 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>156052</v>
+        <v>157889</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1325,17 +1313,639 @@
         <v>46281</v>
       </c>
       <c r="H23" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>72</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>144460</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H24" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>72</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H25" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>47.66</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>72</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>140705</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H26" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>72</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>145423</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H27" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>58.28</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>147</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>141361</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H28" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>72</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>95842</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>46753</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H29" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>72</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>122050</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>46905</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H30" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>49.61</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>72</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>140846</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H31" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>22</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>72</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>151540</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>46569</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H32" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>72</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>152321</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H33" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>72</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>161127</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H34" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>21.12</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>72</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>157926</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H35" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>72</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>142054</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H36" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>72</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>161944</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H37" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>72</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H38" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>147</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H39" t="n">
         <v>789825</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J23" t="n">
+      <c r="J39" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K39" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:15:03
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -792,15 +792,15 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4006</v>
+        <v>123480</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -808,15 +808,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>12.48</v>
+        <v>43.6</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -837,29 +837,23 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>4006</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>31.51</v>
+        <v>12.48</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -880,23 +874,29 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>141092</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G12" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7.29</v>
+        <v>31.51</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>140738</v>
+        <v>141092</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -925,15 +925,15 @@
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>29.12</v>
+        <v>7.29</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -954,29 +954,23 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>140738</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>11.27</v>
+        <v>29.12</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -997,15 +991,15 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>39233</v>
+        <v>148126</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46905</v>
+        <v>46874</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46281</v>
@@ -1019,7 +1013,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>17.83</v>
+        <v>11.27</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1040,23 +1034,29 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>154430</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G16" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H16" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>29.46</v>
+        <v>17.83</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>134701</v>
+        <v>154430</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -1085,15 +1085,15 @@
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>9.35</v>
+        <v>29.46</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>161224</v>
+        <v>141180</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1159,15 +1159,15 @@
         <v>46281</v>
       </c>
       <c r="H19" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>31.97</v>
+        <v>12.8</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>153194</v>
+        <v>161224</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1196,15 +1196,15 @@
         <v>46281</v>
       </c>
       <c r="H20" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>55.4</v>
+        <v>31.97</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>145691</v>
+        <v>153194</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>38.72</v>
+        <v>55.4</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,29 +1262,23 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>145691</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H22" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>12.86</v>
+        <v>38.72</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1305,23 +1299,29 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>157889</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G23" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H23" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>8.33</v>
+        <v>12.86</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>144460</v>
+        <v>157889</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>6.56</v>
+        <v>8.33</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>155058</v>
+        <v>144460</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1387,15 +1387,15 @@
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>47.66</v>
+        <v>6.56</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>140705</v>
+        <v>155058</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>39.98</v>
+        <v>47.66</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>145423</v>
+        <v>140705</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>58.28</v>
+        <v>39.98</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1482,15 +1482,15 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>141361</v>
+        <v>145423</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1498,15 +1498,15 @@
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>33.04</v>
+        <v>58.28</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1519,37 +1519,31 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>141361</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>7.69</v>
+        <v>33.04</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1570,15 +1564,15 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>122050</v>
+        <v>95842</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2519527</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46905</v>
+        <v>46753</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46281</v>
@@ -1592,7 +1586,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>49.61</v>
+        <v>7.69</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1613,15 +1607,15 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>140846</v>
+        <v>122050</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46813</v>
+        <v>46905</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46281</v>
@@ -1635,7 +1629,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>22</v>
+        <v>49.61</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1656,15 +1650,15 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>151540</v>
+        <v>140846</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46569</v>
+        <v>46813</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
@@ -1678,7 +1672,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>12.46</v>
+        <v>22</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1699,23 +1693,29 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>8.83</v>
+        <v>12.46</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>161127</v>
+        <v>152321</v>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
@@ -1744,15 +1744,15 @@
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>21.12</v>
+        <v>8.83</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>157926</v>
+        <v>161127</v>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>22.3</v>
+        <v>21.12</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>142054</v>
+        <v>157926</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>12.8</v>
+        <v>22.3</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1847,29 +1847,23 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>142054</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H37" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>57.06</v>
+        <v>12.8</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1890,23 +1884,29 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>140746</v>
-      </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
+        <v>161944</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G38" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>68.16</v>
+        <v>57.06</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1919,15 +1919,15 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>156052</v>
+        <v>140746</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1935,17 +1935,54 @@
         <v>46281</v>
       </c>
       <c r="H39" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>147</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H40" t="n">
         <v>789825</v>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="J40" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K40" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:30:06
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -866,37 +866,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>149872</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>31.51</v>
+        <v>45.6</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -917,23 +911,29 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>141092</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>7.29</v>
+        <v>31.51</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>140738</v>
+        <v>141092</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -962,15 +962,15 @@
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>29.12</v>
+        <v>7.29</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -991,29 +991,23 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>140738</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H15" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>11.27</v>
+        <v>29.12</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1034,15 +1028,15 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>39233</v>
+        <v>148126</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46905</v>
+        <v>46874</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46281</v>
@@ -1056,7 +1050,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>17.83</v>
+        <v>11.27</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1077,23 +1071,29 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>154430</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G17" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>29.46</v>
+        <v>17.83</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>134701</v>
+        <v>154430</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1122,15 +1122,15 @@
         <v>46281</v>
       </c>
       <c r="H18" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>9.35</v>
+        <v>29.46</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>161224</v>
+        <v>141180</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1196,15 +1196,15 @@
         <v>46281</v>
       </c>
       <c r="H20" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>31.97</v>
+        <v>12.8</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>153194</v>
+        <v>161224</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1233,15 +1233,15 @@
         <v>46281</v>
       </c>
       <c r="H21" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>55.4</v>
+        <v>31.97</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>145691</v>
+        <v>153194</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>38.72</v>
+        <v>55.4</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,29 +1299,23 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>145691</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H23" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>12.86</v>
+        <v>38.72</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1342,23 +1336,29 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>157889</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G24" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H24" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>8.33</v>
+        <v>12.86</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>144460</v>
+        <v>157889</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1395,7 +1395,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>6.56</v>
+        <v>8.33</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>155058</v>
+        <v>144460</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1424,15 +1424,15 @@
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>47.66</v>
+        <v>6.56</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>140705</v>
+        <v>155058</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>39.98</v>
+        <v>47.66</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>145423</v>
+        <v>140705</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>58.28</v>
+        <v>39.98</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1519,15 +1519,15 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>141361</v>
+        <v>145423</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1535,15 +1535,15 @@
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>33.04</v>
+        <v>58.28</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1556,37 +1556,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>141361</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>7.69</v>
+        <v>33.04</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1599,37 +1593,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>49.61</v>
+        <v>198.58</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1650,15 +1638,15 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>140846</v>
+        <v>95842</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>2519527</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46813</v>
+        <v>46753</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
@@ -1672,7 +1660,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>22</v>
+        <v>7.69</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1693,15 +1681,15 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>151540</v>
+        <v>122050</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46569</v>
+        <v>46905</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
@@ -1715,7 +1703,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>12.46</v>
+        <v>49.61</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1736,23 +1724,29 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+        <v>140846</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G34" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>8.83</v>
+        <v>22</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1773,23 +1767,29 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>161127</v>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H35" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>21.12</v>
+        <v>12.46</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>157926</v>
+        <v>152321</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1818,15 +1818,15 @@
         <v>46281</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>22.3</v>
+        <v>8.83</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>142054</v>
+        <v>161127</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>12.8</v>
+        <v>21.12</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1884,29 +1884,23 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>157926</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>57.06</v>
+        <v>22.3</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1927,7 +1921,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>140746</v>
+        <v>142054</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1943,7 +1937,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>68.16</v>
+        <v>12.8</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1956,33 +1950,150 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>72</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>161944</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H40" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>72</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H41" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>142</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H42" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>289.59</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
         <v>147</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D43" t="n">
         <v>156052</v>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H40" t="n">
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H43" t="n">
         <v>789825</v>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J40" t="n">
+      <c r="J43" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K43" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:00:03
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -911,29 +911,23 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>141919</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>33928</v>
+        <v>30307</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>31.51</v>
+        <v>210.43</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -954,7 +948,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>141092</v>
+        <v>156110</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -962,15 +956,15 @@
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>47252</v>
+        <v>30307</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>7.29</v>
+        <v>166.48</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -991,7 +985,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>140738</v>
+        <v>157509</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -999,15 +993,15 @@
         <v>46281</v>
       </c>
       <c r="H15" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>29.12</v>
+        <v>145.61</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1028,29 +1022,29 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>148126</v>
+        <v>140308</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A90B00326</t>
+          <t>2518727</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46874</v>
+        <v>46722</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H16" t="n">
-        <v>31305</v>
+        <v>33928</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>11.27</v>
+        <v>31.51</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1071,29 +1065,23 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>39233</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2606104</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>141092</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>17.83</v>
+        <v>7.29</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1102,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>154430</v>
+        <v>140738</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1122,15 +1110,15 @@
         <v>46281</v>
       </c>
       <c r="H18" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>29.46</v>
+        <v>29.12</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,23 +1139,29 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+        <v>148126</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A90B00326</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G19" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H19" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>9.35</v>
+        <v>11.27</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,23 +1182,29 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>141180</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G20" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H20" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>12.8</v>
+        <v>17.83</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>161224</v>
+        <v>113875</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1233,15 +1233,15 @@
         <v>46281</v>
       </c>
       <c r="H21" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>31.97</v>
+        <v>13.5</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>153194</v>
+        <v>154430</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1270,15 +1270,15 @@
         <v>46281</v>
       </c>
       <c r="H22" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>55.4</v>
+        <v>29.46</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>145691</v>
+        <v>134701</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>38.72</v>
+        <v>9.35</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1336,29 +1336,23 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>141180</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H24" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>12.86</v>
+        <v>12.8</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1379,7 +1373,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>157889</v>
+        <v>163624</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1387,15 +1381,15 @@
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>8.33</v>
+        <v>104.97</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1416,7 +1410,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>144460</v>
+        <v>136630</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1424,15 +1418,15 @@
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>47252</v>
+        <v>30307</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>6.56</v>
+        <v>239.16</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1453,7 +1447,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>155058</v>
+        <v>163047</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1461,15 +1455,15 @@
         <v>46281</v>
       </c>
       <c r="H27" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>47.66</v>
+        <v>226.84</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1490,7 +1484,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>140705</v>
+        <v>161224</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1498,15 +1492,15 @@
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>39.98</v>
+        <v>31.97</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1527,7 +1521,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>145423</v>
+        <v>153194</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1543,7 +1537,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>58.28</v>
+        <v>55.4</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1556,15 +1550,15 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>141361</v>
+        <v>145691</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -1572,15 +1566,15 @@
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>33.04</v>
+        <v>38.72</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1593,31 +1587,37 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>158354</v>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>139553</v>
+        <v>31305</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>198.58</v>
+        <v>12.86</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1638,29 +1638,23 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>162584</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H32" t="n">
-        <v>33928</v>
+        <v>793186</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>7.69</v>
+        <v>103.48</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1681,29 +1675,23 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>157889</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>49.61</v>
+        <v>8.33</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1724,29 +1712,23 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>140846</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2603107</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>144460</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>22</v>
+        <v>6.56</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1767,29 +1749,23 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>155058</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H35" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>12.46</v>
+        <v>47.66</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1810,7 +1786,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>152321</v>
+        <v>140705</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1818,15 +1794,15 @@
         <v>46281</v>
       </c>
       <c r="H36" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>8.83</v>
+        <v>39.98</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1847,7 +1823,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>161127</v>
+        <v>145423</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1863,7 +1839,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>21.12</v>
+        <v>58.28</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1876,15 +1852,15 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>157926</v>
+        <v>141361</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1892,15 +1868,15 @@
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>22.3</v>
+        <v>33.04</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1921,7 +1897,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>142054</v>
+        <v>113883</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1929,15 +1905,15 @@
         <v>46281</v>
       </c>
       <c r="H39" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>12.8</v>
+        <v>13.5</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1950,37 +1926,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H40" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>57.06</v>
+        <v>198.58</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2001,23 +1971,29 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>140746</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+        <v>95842</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G41" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H41" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>68.16</v>
+        <v>7.69</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2030,31 +2006,37 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+        <v>122050</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H42" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>289.59</v>
+        <v>49.61</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2067,33 +2049,458 @@
         </is>
       </c>
       <c r="B43" t="n">
+        <v>72</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>140846</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H43" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>22</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>72</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>151540</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46569</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H44" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>72</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>152321</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H45" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>72</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>161127</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H46" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>21.12</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>72</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>157926</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H47" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>72</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>142054</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H48" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>72</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>84530</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H49" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>48.14</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>72</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>140516</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H50" t="n">
+        <v>30307</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>72</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>161944</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H51" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>72</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H52" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>142</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H53" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>289.59</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
         <v>147</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D54" t="n">
         <v>156052</v>
       </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H43" t="n">
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H54" t="n">
         <v>789825</v>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="J54" t="n">
         <v>67.54000000000001</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K54" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:15:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -496,15 +496,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>70696</v>
+        <v>98221</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -512,15 +512,15 @@
         <v>46281</v>
       </c>
       <c r="H2" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>82.98</v>
+        <v>7.35</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>98221</v>
+        <v>79510</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>7.35</v>
+        <v>8.84</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>79510</v>
+        <v>161738</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>8.84</v>
+        <v>16.79</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>161738</v>
+        <v>143529</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -623,15 +623,15 @@
         <v>46281</v>
       </c>
       <c r="H5" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>16.79</v>
+        <v>21.1</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -652,10 +652,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>143552</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+        <v>155058</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0000281593</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G6" s="2" t="n">
         <v>46281</v>
       </c>
@@ -668,7 +674,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>23.94</v>
+        <v>47.66</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -689,7 +695,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>157169</v>
+        <v>4006</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -705,7 +711,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>23.7</v>
+        <v>12.48</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -718,15 +724,15 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>155062</v>
+        <v>149872</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -742,7 +748,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>63.38</v>
+        <v>45.6</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -755,18 +761,24 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>143529</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+        <v>141361</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A09A06326</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G9" s="2" t="n">
         <v>46281</v>
       </c>
@@ -779,7 +791,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>21.1</v>
+        <v>33.04</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -792,15 +804,15 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>123480</v>
+        <v>141919</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -808,15 +820,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>33928</v>
+        <v>30307</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>43.6</v>
+        <v>210.43</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -837,7 +849,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4006</v>
+        <v>156110</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -845,15 +857,15 @@
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>12.48</v>
+        <v>166.48</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -866,15 +878,15 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>149872</v>
+        <v>157509</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -882,15 +894,15 @@
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>45.6</v>
+        <v>145.61</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -911,23 +923,29 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>141919</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>30307</v>
+        <v>33928</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>210.43</v>
+        <v>31.51</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -948,7 +966,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>156110</v>
+        <v>141092</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -956,15 +974,15 @@
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>166.48</v>
+        <v>7.29</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -985,23 +1003,29 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>157509</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+        <v>155062</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0000293487</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>47119</v>
+      </c>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H15" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>145.61</v>
+        <v>63.38</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1022,29 +1046,29 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>140308</v>
+        <v>140746</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2518727</t>
+          <t>0000291396</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46722</v>
+        <v>46784</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H16" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>31.51</v>
+        <v>68.16</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1065,23 +1089,29 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>141092</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+        <v>161127</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0000293755</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G17" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>7.29</v>
+        <v>21.12</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1102,10 +1132,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+        <v>145691</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0000287662</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>46631</v>
+      </c>
       <c r="G18" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1118,7 +1154,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>29.12</v>
+        <v>38.72</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1299,10 +1335,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+        <v>145423</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0000292962</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G23" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1315,7 +1357,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>9.35</v>
+        <v>58.28</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1336,10 +1378,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>141180</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G24" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1352,7 +1400,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>12.8</v>
+        <v>23.7</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1373,7 +1421,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>163624</v>
+        <v>134701</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1381,15 +1429,15 @@
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>104.97</v>
+        <v>9.35</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1410,7 +1458,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>136630</v>
+        <v>141180</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1418,15 +1466,15 @@
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>239.16</v>
+        <v>12.8</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1447,7 +1495,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>163047</v>
+        <v>163624</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1455,15 +1503,15 @@
         <v>46281</v>
       </c>
       <c r="H27" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>226.84</v>
+        <v>104.97</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1476,31 +1524,37 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>161224</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G28" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>47252</v>
+        <v>789825</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>31.97</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1521,7 +1575,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>153194</v>
+        <v>136630</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1529,15 +1583,15 @@
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>55.4</v>
+        <v>239.16</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1558,7 +1612,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>145691</v>
+        <v>163047</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -1566,15 +1620,15 @@
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>38.72</v>
+        <v>226.84</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1595,29 +1649,23 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>161224</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>12.86</v>
+        <v>31.97</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1638,23 +1686,29 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H32" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>103.48</v>
+        <v>29.12</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1675,23 +1729,29 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>157889</v>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>8.33</v>
+        <v>12.86</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1712,7 +1772,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>144460</v>
+        <v>162584</v>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
@@ -1720,15 +1780,15 @@
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>6.56</v>
+        <v>103.48</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1741,31 +1801,37 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
+        <v>123480</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2517347</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H35" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>47.66</v>
+        <v>43.6</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1786,7 +1852,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>140705</v>
+        <v>157889</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1794,15 +1860,15 @@
         <v>46281</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>39.98</v>
+        <v>8.33</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1823,7 +1889,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>145423</v>
+        <v>144460</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1831,15 +1897,15 @@
         <v>46281</v>
       </c>
       <c r="H37" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>58.28</v>
+        <v>6.56</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1852,15 +1918,15 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>141361</v>
+        <v>113883</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1868,15 +1934,15 @@
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>31305</v>
+        <v>793186</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>33.04</v>
+        <v>13.5</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1889,15 +1955,15 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>113883</v>
+        <v>158354</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1905,15 +1971,15 @@
         <v>46281</v>
       </c>
       <c r="H39" t="n">
-        <v>793186</v>
+        <v>139553</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>13.5</v>
+        <v>198.58</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1926,31 +1992,37 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>158354</v>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
+        <v>95842</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G40" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H40" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>198.58</v>
+        <v>7.69</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -1971,15 +2043,15 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>95842</v>
+        <v>122050</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2519527</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46753</v>
+        <v>46905</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46281</v>
@@ -1993,7 +2065,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>7.69</v>
+        <v>49.61</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2014,15 +2086,15 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>122050</v>
+        <v>140846</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46905</v>
+        <v>46813</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
@@ -2036,7 +2108,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>49.61</v>
+        <v>22</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2057,15 +2129,15 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>140846</v>
+        <v>151540</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>20012026</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46813</v>
+        <v>46569</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46281</v>
@@ -2079,7 +2151,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>22</v>
+        <v>12.46</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2100,29 +2172,23 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>152321</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>12.46</v>
+        <v>8.83</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2143,7 +2209,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>152321</v>
+        <v>157926</v>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
@@ -2151,15 +2217,15 @@
         <v>46281</v>
       </c>
       <c r="H45" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8.83</v>
+        <v>22.3</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2180,7 +2246,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>161127</v>
+        <v>142054</v>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
@@ -2196,7 +2262,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>21.12</v>
+        <v>12.8</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2217,7 +2283,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>157926</v>
+        <v>84530</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
@@ -2225,15 +2291,15 @@
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>22.3</v>
+        <v>48.14</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2254,7 +2320,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>142054</v>
+        <v>140516</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
@@ -2262,15 +2328,15 @@
         <v>46281</v>
       </c>
       <c r="H48" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>12.8</v>
+        <v>108.8</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2291,23 +2357,29 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>84530</v>
-      </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+        <v>161944</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H49" t="n">
-        <v>793186</v>
+        <v>33928</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>48.14</v>
+        <v>57.06</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2320,31 +2392,37 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>140516</v>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+        <v>70696</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2605007</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G50" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H50" t="n">
-        <v>30307</v>
+        <v>33928</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>108.8</v>
+        <v>82.98</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2365,29 +2443,29 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>161944</v>
+        <v>140705</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2514837</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46813</v>
+        <v>46844</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H51" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>57.06</v>
+        <v>39.98</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2408,10 +2486,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>140746</v>
-      </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
+        <v>153194</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>46508</v>
+      </c>
       <c r="G52" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2424,7 +2508,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>68.16</v>
+        <v>55.4</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2437,18 +2521,24 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G53" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2461,7 +2551,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>289.59</v>
+        <v>23.94</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2474,15 +2564,15 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>156052</v>
+        <v>155058</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2490,15 +2580,15 @@
         <v>46281</v>
       </c>
       <c r="H54" t="n">
-        <v>789825</v>
+        <v>789423</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>67.54000000000001</v>
+        <v>289.59</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:30:03
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,15 +496,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>98221</v>
+        <v>140760</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -512,15 +512,15 @@
         <v>46281</v>
       </c>
       <c r="H2" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>7.35</v>
+        <v>116.48</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -533,15 +533,15 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>79510</v>
+        <v>153194</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -549,15 +549,15 @@
         <v>46281</v>
       </c>
       <c r="H3" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>8.84</v>
+        <v>105.98</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -570,15 +570,15 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>161738</v>
+        <v>139483</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -586,15 +586,15 @@
         <v>46281</v>
       </c>
       <c r="H4" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>16.79</v>
+        <v>156.3</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -607,15 +607,15 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>143529</v>
+        <v>154914</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -623,15 +623,15 @@
         <v>46281</v>
       </c>
       <c r="H5" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>21.1</v>
+        <v>128.63</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -644,24 +644,18 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0000281593</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>134701</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" s="2" t="n">
         <v>46281</v>
       </c>
@@ -674,7 +668,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>47.66</v>
+        <v>74.73</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -687,15 +681,15 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4006</v>
+        <v>143551</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -711,7 +705,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>12.48</v>
+        <v>106.92</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -732,7 +726,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>149872</v>
+        <v>140705</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -748,7 +742,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>45.6</v>
+        <v>171</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -761,37 +755,31 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>A09A06326</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>140717</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H9" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>33.04</v>
+        <v>117.56</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -812,7 +800,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>141919</v>
+        <v>143529</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -820,15 +808,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>30307</v>
+        <v>31305</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>210.43</v>
+        <v>21.1</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -849,23 +837,29 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>156110</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+        <v>98221</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B25H1859</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>46600</v>
+      </c>
       <c r="G11" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>166.48</v>
+        <v>7.35</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -886,23 +880,29 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>157509</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+        <v>144460</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B26E0774</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G12" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>145.61</v>
+        <v>6.56</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -923,29 +923,29 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>140308</v>
+        <v>155058</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2518727</t>
+          <t>0000281593</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46722</v>
+        <v>46569</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>31.51</v>
+        <v>47.66</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>141092</v>
+        <v>4006</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -974,15 +974,15 @@
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>7.29</v>
+        <v>12.48</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -995,24 +995,18 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>155062</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>0000293487</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>47119</v>
-      </c>
+        <v>140719</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1025,7 +1019,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>63.38</v>
+        <v>214.71</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1038,24 +1032,18 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>140746</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>0000291396</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>46784</v>
-      </c>
+        <v>142054</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1068,7 +1056,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>68.16</v>
+        <v>57.15</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1081,24 +1069,18 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>161127</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0000293755</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>105481</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1111,7 +1093,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>21.12</v>
+        <v>486.57</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1124,24 +1106,18 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>145691</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>0000287662</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>46631</v>
-      </c>
+        <v>143382</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1154,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>38.72</v>
+        <v>238.04</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1167,37 +1143,31 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>8451</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H19" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>11.27</v>
+        <v>311.01</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1210,37 +1180,31 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>39233</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2606104</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>128896</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H20" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>17.83</v>
+        <v>118.12</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1253,15 +1217,15 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>113875</v>
+        <v>155062</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1269,15 +1233,15 @@
         <v>46281</v>
       </c>
       <c r="H21" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>13.5</v>
+        <v>2311.03</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1290,15 +1254,15 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>154430</v>
+        <v>1600</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1306,15 +1270,15 @@
         <v>46281</v>
       </c>
       <c r="H22" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>29.46</v>
+        <v>121.72</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1327,24 +1291,18 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>145423</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0000292962</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>149872</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1357,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>58.28</v>
+        <v>45.6</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1370,37 +1328,37 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>157169</v>
+        <v>141361</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>A09A06326</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46753</v>
+        <v>46905</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H24" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>23.7</v>
+        <v>33.04</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1421,7 +1379,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>134701</v>
+        <v>141919</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1429,15 +1387,15 @@
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>9.35</v>
+        <v>210.43</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1458,7 +1416,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>141180</v>
+        <v>156110</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1466,15 +1424,15 @@
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>12.8</v>
+        <v>166.48</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1495,7 +1453,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>163624</v>
+        <v>157509</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1503,15 +1461,15 @@
         <v>46281</v>
       </c>
       <c r="H27" t="n">
-        <v>793186</v>
+        <v>30307</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>104.97</v>
+        <v>145.61</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1524,37 +1482,31 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>162951</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>789825</v>
+        <v>796770</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>67.54000000000001</v>
+        <v>155.18</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1575,23 +1527,29 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>136630</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G29" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>30307</v>
+        <v>33928</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>239.16</v>
+        <v>31.51</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1612,23 +1570,29 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>163047</v>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+        <v>161738</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>B26B1405</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>46784</v>
+      </c>
       <c r="G30" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>226.84</v>
+        <v>16.79</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1649,23 +1613,29 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>161224</v>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+        <v>155062</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0000293487</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>47119</v>
+      </c>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>31.97</v>
+        <v>63.38</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1686,15 +1656,15 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>140738</v>
+        <v>140746</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0000289599</t>
+          <t>0000291396</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46661</v>
+        <v>46784</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
@@ -1708,7 +1678,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>29.12</v>
+        <v>68.16</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1729,29 +1699,29 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>12521</v>
+        <v>161127</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A44A00626</t>
+          <t>0000293755</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46844</v>
+        <v>46753</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>12.86</v>
+        <v>21.12</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1772,23 +1742,29 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+        <v>145691</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0000287662</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>46631</v>
+      </c>
       <c r="G34" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>103.48</v>
+        <v>38.72</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1801,37 +1777,31 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>127998</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H35" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>43.6</v>
+        <v>162.79</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1844,15 +1814,15 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>157889</v>
+        <v>162453</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1860,15 +1830,15 @@
         <v>46281</v>
       </c>
       <c r="H36" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>8.33</v>
+        <v>151.35</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1881,15 +1851,15 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>144460</v>
+        <v>146046</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1897,15 +1867,15 @@
         <v>46281</v>
       </c>
       <c r="H37" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>6.56</v>
+        <v>112.87</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1918,15 +1888,15 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>113883</v>
+        <v>159926</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1934,15 +1904,15 @@
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>13.5</v>
+        <v>186.19</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1955,15 +1925,15 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>158354</v>
+        <v>140745</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1971,15 +1941,15 @@
         <v>46281</v>
       </c>
       <c r="H39" t="n">
-        <v>139553</v>
+        <v>789423</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>198.58</v>
+        <v>832.27</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1992,37 +1962,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>147555</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H40" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>7.69</v>
+        <v>552.17</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2035,37 +1999,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H41" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>49.61</v>
+        <v>242.61</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2086,29 +2044,29 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>140846</v>
+        <v>148126</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46813</v>
+        <v>46874</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H42" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>22</v>
+        <v>11.27</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2129,29 +2087,29 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>151540</v>
+        <v>39233</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2606104</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46569</v>
+        <v>46905</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H43" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>12.46</v>
+        <v>17.83</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2172,7 +2130,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>152321</v>
+        <v>113875</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
@@ -2180,15 +2138,15 @@
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>8.83</v>
+        <v>13.5</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2209,23 +2167,29 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>157926</v>
-      </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
+        <v>152321</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>B26E1180</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G45" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H45" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>22.3</v>
+        <v>8.83</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2246,23 +2210,29 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>142054</v>
-      </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
+        <v>141092</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>B26E1386</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G46" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H46" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>12.8</v>
+        <v>7.29</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2283,23 +2253,29 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>84530</v>
-      </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
+        <v>157889</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2502015</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G47" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>48.14</v>
+        <v>8.33</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2320,23 +2296,29 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>140516</v>
-      </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
+        <v>145423</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0000292962</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G48" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H48" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>108.8</v>
+        <v>58.28</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2357,29 +2339,29 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>161944</v>
+        <v>157169</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2514837</t>
+          <t>0000294775</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46813</v>
+        <v>46753</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H49" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>57.06</v>
+        <v>23.7</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2392,37 +2374,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>70696</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2605007</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>134701</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H50" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>82.98</v>
+        <v>9.35</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2443,16 +2419,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>140705</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>0000301524</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>141180</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2465,7 +2435,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>39.98</v>
+        <v>12.8</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2478,24 +2448,18 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>153194</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>0000297125</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>46508</v>
-      </c>
+        <v>66656</v>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2508,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>55.4</v>
+        <v>32.66</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2521,24 +2485,18 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>143552</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>0000289416</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>140753</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2551,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>23.94</v>
+        <v>118.12</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2572,7 +2530,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>155058</v>
+        <v>143381</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2588,9 +2546,2177 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>289.59</v>
+        <v>183.68</v>
       </c>
       <c r="K54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>142</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>140709</v>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H55" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>165.61</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>142</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>140718</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H56" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>213.72</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>142</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>141180</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H57" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>142</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>22098</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H58" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>62.47</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>142</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>46728</v>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H59" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>249.78</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>72</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>163624</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H60" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>104.97</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>147</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>156052</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>46753</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H61" t="n">
+        <v>789825</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>67.54000000000001</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>72</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>136630</v>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H62" t="n">
+        <v>30307</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>239.16</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>72</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>163047</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H63" t="n">
+        <v>30307</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>226.84</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>72</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>140738</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>46661</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H64" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>29.12</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>142</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>143384</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H65" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>653.86</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>142</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>140710</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H66" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>75.84</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>142</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>105546</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H67" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>806.15</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>142</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>155959</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H68" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>65.31999999999999</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>72</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>12521</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>46844</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H69" t="n">
+        <v>31305</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>LABORATORIO GLOBO LTDA</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>72</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>162584</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H70" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>103.48</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>147</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>123480</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2517347</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>46692</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H71" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>72</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>79510</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>B26C2880</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>46844</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H72" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>161224</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>B26F1555</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>46905</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H73" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>31.97</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>142</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>145623</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H74" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>52.18</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>142</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>162452</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H75" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>106.11</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>142</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>142053</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H76" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>142</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>142886</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H77" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>54.88</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>142</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1120</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H78" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>79.27</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>142</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>27723</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H79" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>385.19</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>72</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>113883</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H80" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>135</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>158354</v>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H81" t="n">
+        <v>139553</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>198.58</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>72</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>95842</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>46753</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H82" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>72</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>122050</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>46905</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H83" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>49.61</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>72</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>140846</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H84" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>22</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>72</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>151540</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>46569</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H85" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>72</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>157926</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H86" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>72</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>142054</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H87" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>142</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>4006</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H88" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>106.69</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>142</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>105236</v>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H89" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>770.38</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>142</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>145757</v>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H90" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>128.22</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>142</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>105465</v>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H91" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>142</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>105511</v>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H92" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>62.47</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>142</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>105490</v>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H93" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>246.9</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>72</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>84530</v>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H94" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>48.14</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>72</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>140516</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H95" t="n">
+        <v>30307</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>135</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>162989</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H96" t="n">
+        <v>796770</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>155.18</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>72</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>161944</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>46813</v>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H97" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>57.06</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>147</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>70696</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2605007</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>46844</v>
+      </c>
+      <c r="G98" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H98" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>82.98</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>72</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>154430</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>NEG02225</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>46692</v>
+      </c>
+      <c r="G99" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H99" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>HYPERA S.A</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>29.46</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>72</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>140705</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>0000301524</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>46844</v>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H100" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>72</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>153194</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H101" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>72</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>DIRETORIA KA BETA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>143552</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>46661</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H102" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>23.94</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>142</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>141811</v>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H103" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>107.64</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>142</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>162443</v>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H104" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>220.91</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>142</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H105" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>482.65</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>142</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>2283</v>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H106" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>318.34</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>142</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>7226</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H107" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>293.44</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>142</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>105228</v>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H108" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>2753.62</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>142</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>145423</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H109" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>257.04</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>142</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>140716</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H110" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>113.25</v>
+      </c>
+      <c r="K110" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:45:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>147555</v>
+        <v>105600</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>552.17</v>
+        <v>242.61</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -1999,31 +1999,37 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>105600</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+        <v>148126</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>A90B00326</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G41" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H41" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>242.61</v>
+        <v>11.27</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2044,15 +2050,15 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>148126</v>
+        <v>39233</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>A90B00326</t>
+          <t>2606104</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46874</v>
+        <v>46905</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
@@ -2066,7 +2072,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>11.27</v>
+        <v>17.83</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2087,29 +2093,23 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>39233</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2606104</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>113875</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H43" t="n">
-        <v>31305</v>
+        <v>793186</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>17.83</v>
+        <v>13.5</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2130,23 +2130,29 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>113875</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
+        <v>152321</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>B26E1180</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G44" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>13.5</v>
+        <v>8.83</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2167,15 +2173,15 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>152321</v>
+        <v>141092</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>B26E1180</t>
+          <t>B26E1386</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46813</v>
+        <v>46874</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46281</v>
@@ -2189,7 +2195,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8.83</v>
+        <v>7.29</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2210,15 +2216,15 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>141092</v>
+        <v>157889</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>B26E1386</t>
+          <t>2502015</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46874</v>
+        <v>46844</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46281</v>
@@ -2232,7 +2238,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>7.29</v>
+        <v>8.33</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2253,29 +2259,29 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>157889</v>
+        <v>145423</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2502015</t>
+          <t>0000292962</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46844</v>
+        <v>46753</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>8.33</v>
+        <v>58.28</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2296,11 +2302,11 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>145423</v>
+        <v>157169</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000292962</t>
+          <t>0000294775</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -2318,7 +2324,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>58.28</v>
+        <v>23.7</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2339,16 +2345,10 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>157169</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>0000294775</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>134701</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>23.7</v>
+        <v>9.35</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134701</v>
+        <v>141180</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>9.35</v>
+        <v>12.8</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2411,15 +2411,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>141180</v>
+        <v>66656</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>12.8</v>
+        <v>32.66</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>66656</v>
+        <v>140753</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>32.66</v>
+        <v>118.12</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>140753</v>
+        <v>143381</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>118.12</v>
+        <v>183.68</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>143381</v>
+        <v>140709</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>183.68</v>
+        <v>165.61</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>140709</v>
+        <v>140718</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>165.61</v>
+        <v>213.72</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>140718</v>
+        <v>141180</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>213.72</v>
+        <v>57.15</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>141180</v>
+        <v>22098</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>57.15</v>
+        <v>62.47</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>22098</v>
+        <v>46728</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>62.47</v>
+        <v>249.78</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2707,15 +2707,15 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>46728</v>
+        <v>163624</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
@@ -2723,15 +2723,15 @@
         <v>46281</v>
       </c>
       <c r="H59" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>249.78</v>
+        <v>104.97</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2744,31 +2744,37 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>163624</v>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G60" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H60" t="n">
-        <v>793186</v>
+        <v>789825</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>104.97</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2781,37 +2787,31 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>136630</v>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H61" t="n">
-        <v>789825</v>
+        <v>30307</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>67.54000000000001</v>
+        <v>239.16</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2832,7 +2832,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>136630</v>
+        <v>163047</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2848,7 +2848,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>239.16</v>
+        <v>226.84</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2869,23 +2869,29 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>163047</v>
-      </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G63" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H63" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>226.84</v>
+        <v>29.12</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2898,24 +2904,18 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>0000289599</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>143384</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2928,7 +2928,7 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>29.12</v>
+        <v>653.86</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>143384</v>
+        <v>140710</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>653.86</v>
+        <v>75.84</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>140710</v>
+        <v>105546</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>75.84</v>
+        <v>806.15</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>105546</v>
+        <v>155959</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>806.15</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3052,31 +3052,37 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>155959</v>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G68" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H68" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>65.31999999999999</v>
+        <v>12.86</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3097,29 +3103,23 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>162584</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H69" t="n">
-        <v>31305</v>
+        <v>793186</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>12.86</v>
+        <v>103.48</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3132,31 +3132,37 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
+        <v>123480</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2517347</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G70" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H70" t="n">
-        <v>793186</v>
+        <v>33928</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>103.48</v>
+        <v>43.6</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3169,37 +3175,37 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>123480</v>
+        <v>79510</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2517347</t>
+          <t>B26C2880</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46692</v>
+        <v>46844</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H71" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>43.6</v>
+        <v>8.84</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3220,15 +3226,15 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>79510</v>
+        <v>161224</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>B26F1555</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>46844</v>
+        <v>46905</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>46281</v>
@@ -3242,7 +3248,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>8.84</v>
+        <v>31.97</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3255,37 +3261,31 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>161224</v>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>B26F1555</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>145623</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H73" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>31.97</v>
+        <v>52.18</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>145623</v>
+        <v>162452</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
@@ -3322,7 +3322,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>52.18</v>
+        <v>106.11</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>162452</v>
+        <v>142053</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>106.11</v>
+        <v>57.15</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3380,7 +3380,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>142053</v>
+        <v>142886</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
@@ -3396,7 +3396,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>57.15</v>
+        <v>54.88</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>142886</v>
+        <v>1120</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>54.88</v>
+        <v>79.27</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1120</v>
+        <v>27723</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>79.27</v>
+        <v>385.19</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3483,15 +3483,15 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>27723</v>
+        <v>113883</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3499,15 +3499,15 @@
         <v>46281</v>
       </c>
       <c r="H79" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>385.19</v>
+        <v>13.5</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3520,15 +3520,15 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>113883</v>
+        <v>158354</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3536,15 +3536,15 @@
         <v>46281</v>
       </c>
       <c r="H80" t="n">
-        <v>793186</v>
+        <v>139553</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>13.5</v>
+        <v>198.58</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3557,31 +3557,37 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>158354</v>
-      </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
+        <v>95842</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G81" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H81" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>198.58</v>
+        <v>7.69</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3602,15 +3608,15 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>95842</v>
+        <v>122050</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2519527</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>46753</v>
+        <v>46905</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>46281</v>
@@ -3624,7 +3630,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>7.69</v>
+        <v>49.61</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3645,15 +3651,15 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>122050</v>
+        <v>140846</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>46905</v>
+        <v>46813</v>
       </c>
       <c r="G83" s="2" t="n">
         <v>46281</v>
@@ -3667,7 +3673,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>49.61</v>
+        <v>22</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3688,15 +3694,15 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>140846</v>
+        <v>151540</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>20012026</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>46813</v>
+        <v>46569</v>
       </c>
       <c r="G84" s="2" t="n">
         <v>46281</v>
@@ -3710,7 +3716,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>22</v>
+        <v>12.46</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3731,29 +3737,23 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>157926</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>12.46</v>
+        <v>22.3</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>157926</v>
+        <v>142054</v>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
@@ -3790,7 +3790,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>22.3</v>
+        <v>12.8</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3803,15 +3803,15 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>142054</v>
+        <v>4006</v>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>12.8</v>
+        <v>106.69</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3848,7 +3848,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>4006</v>
+        <v>105236</v>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
@@ -3864,7 +3864,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>106.69</v>
+        <v>770.38</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>105236</v>
+        <v>145757</v>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>770.38</v>
+        <v>128.22</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>145757</v>
+        <v>105465</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
@@ -3938,7 +3938,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>128.22</v>
+        <v>96.3</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>105465</v>
+        <v>105511</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>96.3</v>
+        <v>62.47</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>105511</v>
+        <v>105490</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>62.47</v>
+        <v>246.9</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4025,15 +4025,15 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>105490</v>
+        <v>84530</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4041,15 +4041,15 @@
         <v>46281</v>
       </c>
       <c r="H93" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>246.9</v>
+        <v>48.14</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>84530</v>
+        <v>140516</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4078,15 +4078,15 @@
         <v>46281</v>
       </c>
       <c r="H94" t="n">
-        <v>793186</v>
+        <v>30307</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>48.14</v>
+        <v>108.8</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4099,15 +4099,15 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>140516</v>
+        <v>162989</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4115,15 +4115,15 @@
         <v>46281</v>
       </c>
       <c r="H95" t="n">
-        <v>30307</v>
+        <v>796770</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>108.8</v>
+        <v>155.18</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4136,31 +4136,37 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>162989</v>
-      </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
+        <v>161944</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G96" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H96" t="n">
-        <v>796770</v>
+        <v>33928</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>155.18</v>
+        <v>57.06</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4173,23 +4179,23 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>161944</v>
+        <v>70696</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2514837</t>
+          <t>2605007</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>46813</v>
+        <v>46844</v>
       </c>
       <c r="G97" s="2" t="n">
         <v>46281</v>
@@ -4203,7 +4209,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>57.06</v>
+        <v>82.98</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4216,37 +4222,37 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>70696</v>
+        <v>154430</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2605007</t>
+          <t>NEG02225</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G98" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H98" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>82.98</v>
+        <v>29.46</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4267,29 +4273,29 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>154430</v>
+        <v>140705</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>NEG02225</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>46692</v>
+        <v>46844</v>
       </c>
       <c r="G99" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H99" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>29.46</v>
+        <v>39.98</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4310,15 +4316,15 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>140705</v>
+        <v>153194</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>0000301524</t>
+          <t>0000297125</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>46844</v>
+        <v>46508</v>
       </c>
       <c r="G100" s="2" t="n">
         <v>46281</v>
@@ -4332,7 +4338,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>39.98</v>
+        <v>55.4</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4353,15 +4359,15 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>153194</v>
+        <v>143552</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>0000297125</t>
+          <t>0000289416</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>46508</v>
+        <v>46661</v>
       </c>
       <c r="G101" s="2" t="n">
         <v>46281</v>
@@ -4375,7 +4381,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>55.4</v>
+        <v>23.94</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4388,24 +4394,18 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>143552</v>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>0000289416</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>141811</v>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4418,7 +4418,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>23.94</v>
+        <v>107.64</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4439,7 +4439,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>141811</v>
+        <v>162443</v>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>107.64</v>
+        <v>220.91</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4476,7 +4476,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>162443</v>
+        <v>155058</v>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>220.91</v>
+        <v>482.65</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>155058</v>
+        <v>2283</v>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
@@ -4529,7 +4529,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>482.65</v>
+        <v>318.34</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>2283</v>
+        <v>7226</v>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>318.34</v>
+        <v>293.44</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>7226</v>
+        <v>105228</v>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>293.44</v>
+        <v>2753.62</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4624,7 +4624,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>105228</v>
+        <v>145423</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>2753.62</v>
+        <v>257.04</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>145423</v>
+        <v>140716</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
@@ -4677,46 +4677,9 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>257.04</v>
+        <v>113.25</v>
       </c>
       <c r="K109" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B110" t="n">
-        <v>142</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
-        </is>
-      </c>
-      <c r="D110" t="n">
-        <v>140716</v>
-      </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H110" t="n">
-        <v>789423</v>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
-        </is>
-      </c>
-      <c r="J110" t="n">
-        <v>113.25</v>
-      </c>
-      <c r="K110" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 12:27:14
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,15 +496,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>140760</v>
+        <v>105228</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>116.48</v>
+        <v>84.3</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>153194</v>
+        <v>140760</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>105.98</v>
+        <v>291.2</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>139483</v>
+        <v>153194</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>156.3</v>
+        <v>741.89</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>154914</v>
+        <v>139483</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>128.63</v>
+        <v>156.3</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>134701</v>
+        <v>154914</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>74.73</v>
+        <v>128.63</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>143551</v>
+        <v>134701</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>106.92</v>
+        <v>74.73</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>140705</v>
+        <v>143551</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>171</v>
+        <v>106.92</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>140717</v>
+        <v>140705</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>117.56</v>
+        <v>342</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -792,15 +792,15 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>143529</v>
+        <v>140717</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -808,15 +808,15 @@
         <v>46281</v>
       </c>
       <c r="H10" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>21.1</v>
+        <v>117.56</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -837,29 +837,23 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>98221</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>B25H1859</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>46600</v>
-      </c>
+        <v>143529</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H11" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>7.35</v>
+        <v>21.1</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -880,15 +874,15 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>144460</v>
+        <v>98221</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B26E0774</t>
+          <t>B25H1859</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46874</v>
+        <v>46600</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46281</v>
@@ -902,7 +896,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>6.56</v>
+        <v>7.35</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -923,29 +917,29 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>155058</v>
+        <v>144460</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0000281593</t>
+          <t>B26E0774</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46569</v>
+        <v>46874</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>47.66</v>
+        <v>6.56</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -966,10 +960,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4006</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+        <v>155058</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0000281593</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G14" s="2" t="n">
         <v>46281</v>
       </c>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>12.48</v>
+        <v>47.66</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -995,15 +995,15 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>140719</v>
+        <v>4006</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>214.71</v>
+        <v>12.48</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>142054</v>
+        <v>140719</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>57.15</v>
+        <v>214.71</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>105481</v>
+        <v>8451</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>486.57</v>
+        <v>435.41</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>143382</v>
+        <v>142054</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>238.04</v>
+        <v>271.48</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8451</v>
+        <v>105481</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>311.01</v>
+        <v>973.14</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>128896</v>
+        <v>143382</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>118.12</v>
+        <v>238.04</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>155062</v>
+        <v>128896</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>2311.03</v>
+        <v>118.12</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1600</v>
+        <v>155062</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>121.72</v>
+        <v>2311.03</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>149872</v>
+        <v>1600</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>45.6</v>
+        <v>121.72</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1328,37 +1328,31 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>A09A06326</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>149872</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H24" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>33.04</v>
+        <v>45.6</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1371,31 +1365,37 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>141919</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+        <v>141361</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A09A06326</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G25" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>30307</v>
+        <v>31305</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>210.43</v>
+        <v>33.04</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>156110</v>
+        <v>141919</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>166.48</v>
+        <v>210.43</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>157509</v>
+        <v>156110</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>145.61</v>
+        <v>166.48</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1482,15 +1482,15 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>162951</v>
+        <v>157509</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1498,15 +1498,15 @@
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>155.18</v>
+        <v>145.61</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1519,37 +1519,31 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>162951</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>31.51</v>
+        <v>155.18</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1570,29 +1564,29 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>161738</v>
+        <v>140308</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>B26B1405</t>
+          <t>2518727</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46784</v>
+        <v>46722</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>16.79</v>
+        <v>31.51</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1613,29 +1607,29 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>155062</v>
+        <v>161738</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0000293487</t>
+          <t>B26B1405</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>47119</v>
+        <v>46784</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>63.38</v>
+        <v>16.79</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1656,15 +1650,15 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>140746</v>
+        <v>155062</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0000291396</t>
+          <t>0000293487</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46784</v>
+        <v>47119</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
@@ -1678,7 +1672,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>68.16</v>
+        <v>63.38</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1699,15 +1693,15 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>161127</v>
+        <v>140746</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0000293755</t>
+          <t>0000291396</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46753</v>
+        <v>46784</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
@@ -1721,7 +1715,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>21.12</v>
+        <v>68.16</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1742,15 +1736,15 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>145691</v>
+        <v>161127</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0000287662</t>
+          <t>0000293755</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46631</v>
+        <v>46753</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46281</v>
@@ -1764,7 +1758,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>38.72</v>
+        <v>21.12</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1777,18 +1771,24 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>127998</v>
-      </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
+        <v>145691</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0000287662</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>46631</v>
+      </c>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>162.79</v>
+        <v>38.72</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>162453</v>
+        <v>127998</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>151.35</v>
+        <v>651.15</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>146046</v>
+        <v>162453</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>112.87</v>
+        <v>151.35</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>159926</v>
+        <v>146046</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>186.19</v>
+        <v>112.87</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>140745</v>
+        <v>159926</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>832.27</v>
+        <v>248.25</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>105600</v>
+        <v>140745</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>242.61</v>
+        <v>1248.4</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -1999,37 +1999,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H41" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>11.27</v>
+        <v>242.61</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2050,15 +2044,15 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>39233</v>
+        <v>148126</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46905</v>
+        <v>46874</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
@@ -2072,7 +2066,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>17.83</v>
+        <v>11.27</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2093,23 +2087,29 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>113875</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G43" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H43" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>13.5</v>
+        <v>17.83</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2130,29 +2130,23 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>B26E1180</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>113875</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>8.83</v>
+        <v>13.5</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2173,15 +2167,15 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>141092</v>
+        <v>152321</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>B26E1386</t>
+          <t>B26E1180</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46874</v>
+        <v>46813</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46281</v>
@@ -2195,7 +2189,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>7.29</v>
+        <v>8.83</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2216,15 +2210,15 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>157889</v>
+        <v>141092</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2502015</t>
+          <t>B26E1386</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46844</v>
+        <v>46874</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46281</v>
@@ -2238,7 +2232,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>8.33</v>
+        <v>7.29</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2259,29 +2253,29 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>145423</v>
+        <v>157889</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0000292962</t>
+          <t>2502015</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46753</v>
+        <v>46844</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>58.28</v>
+        <v>8.33</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2302,11 +2296,11 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>157169</v>
+        <v>145423</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>0000292962</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -2324,7 +2318,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>23.7</v>
+        <v>58.28</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2345,10 +2339,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>9.35</v>
+        <v>23.7</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2411,15 +2411,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>66656</v>
+        <v>141180</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>32.66</v>
+        <v>12.8</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>140753</v>
+        <v>141180</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>118.12</v>
+        <v>271.48</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>143381</v>
+        <v>66656</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>183.68</v>
+        <v>236.76</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>140709</v>
+        <v>140753</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>165.61</v>
+        <v>118.12</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>213.72</v>
+        <v>427.44</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>141180</v>
+        <v>143381</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>57.15</v>
+        <v>367.36</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>22098</v>
+        <v>140709</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>62.47</v>
+        <v>165.61</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>46728</v>
+        <v>22098</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>249.78</v>
+        <v>62.47</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2707,15 +2707,15 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>163624</v>
+        <v>46728</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
@@ -2723,15 +2723,15 @@
         <v>46281</v>
       </c>
       <c r="H59" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>104.97</v>
+        <v>333.04</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2744,37 +2744,31 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>157574</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H60" t="n">
-        <v>789825</v>
+        <v>789423</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>67.54000000000001</v>
+        <v>483.7</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2787,15 +2781,15 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>136630</v>
+        <v>143553</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
@@ -2803,15 +2797,15 @@
         <v>46281</v>
       </c>
       <c r="H61" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>239.16</v>
+        <v>424.78</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2832,7 +2826,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>163047</v>
+        <v>163624</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2840,15 +2834,15 @@
         <v>46281</v>
       </c>
       <c r="H62" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>226.84</v>
+        <v>104.97</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2861,37 +2855,37 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>140738</v>
+        <v>156052</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0000289599</t>
+          <t>26A0272</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>46661</v>
+        <v>46753</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H63" t="n">
-        <v>789423</v>
+        <v>789825</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>29.12</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2904,15 +2898,15 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>143384</v>
+        <v>136630</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -2920,15 +2914,15 @@
         <v>46281</v>
       </c>
       <c r="H64" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>653.86</v>
+        <v>239.16</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2941,15 +2935,15 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>140710</v>
+        <v>163047</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2957,15 +2951,15 @@
         <v>46281</v>
       </c>
       <c r="H65" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>75.84</v>
+        <v>226.84</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2978,18 +2972,24 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>105546</v>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G66" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>806.15</v>
+        <v>29.12</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>155959</v>
+        <v>143384</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>65.31999999999999</v>
+        <v>653.86</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3052,37 +3052,31 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>140710</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H68" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>12.86</v>
+        <v>549.87</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3095,15 +3089,15 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>162584</v>
+        <v>105546</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
@@ -3111,15 +3105,15 @@
         <v>46281</v>
       </c>
       <c r="H69" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>103.48</v>
+        <v>959.7</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3132,37 +3126,31 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>155959</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H70" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>43.6</v>
+        <v>310.29</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3183,11 +3171,11 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>79510</v>
+        <v>12521</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>A44A00626</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
@@ -3197,15 +3185,15 @@
         <v>46281</v>
       </c>
       <c r="H71" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>8.84</v>
+        <v>12.86</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3226,29 +3214,23 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>161224</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>B26F1555</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>162584</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H72" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>31.97</v>
+        <v>103.48</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3261,15 +3243,15 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>145623</v>
+        <v>84026</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
@@ -3277,15 +3259,15 @@
         <v>46281</v>
       </c>
       <c r="H73" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>52.18</v>
+        <v>81.25</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3298,31 +3280,37 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>162452</v>
-      </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
+        <v>123480</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2517347</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G74" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H74" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>106.11</v>
+        <v>43.6</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3335,31 +3323,37 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>142053</v>
-      </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
+        <v>79510</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>B26C2880</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G75" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H75" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>57.15</v>
+        <v>8.84</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3372,31 +3366,37 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>142886</v>
-      </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
+        <v>161224</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>B26F1555</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G76" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H76" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>54.88</v>
+        <v>31.97</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1120</v>
+        <v>142053</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>79.27</v>
+        <v>271.48</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>27723</v>
+        <v>145623</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>385.19</v>
+        <v>208.71</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3483,15 +3483,15 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>113883</v>
+        <v>162452</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3499,15 +3499,15 @@
         <v>46281</v>
       </c>
       <c r="H79" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>13.5</v>
+        <v>212.22</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3520,15 +3520,15 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>158354</v>
+        <v>142886</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3536,15 +3536,15 @@
         <v>46281</v>
       </c>
       <c r="H80" t="n">
-        <v>139553</v>
+        <v>789423</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>198.58</v>
+        <v>54.88</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3557,37 +3557,31 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>1120</v>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H81" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>7.69</v>
+        <v>237.8</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3600,37 +3594,31 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>27723</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H82" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>49.61</v>
+        <v>385.19</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3651,29 +3639,23 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>140846</v>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>2603107</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>113883</v>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H83" t="n">
-        <v>33928</v>
+        <v>793186</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>22</v>
+        <v>13.5</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3686,37 +3668,31 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H84" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>12.46</v>
+        <v>198.58</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3737,23 +3713,29 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>157926</v>
-      </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
+        <v>95842</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G85" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>22.3</v>
+        <v>7.69</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3774,23 +3756,29 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>142054</v>
-      </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
+        <v>122050</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G86" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H86" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>12.8</v>
+        <v>49.61</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3803,31 +3791,37 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>4006</v>
-      </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
+        <v>140846</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G87" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H87" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>106.69</v>
+        <v>22</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3840,31 +3834,37 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>105236</v>
-      </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G88" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H88" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>770.38</v>
+        <v>12.46</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3877,15 +3877,15 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>145757</v>
+        <v>157926</v>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>128.22</v>
+        <v>22.3</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3914,15 +3914,15 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>105465</v>
+        <v>142054</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
@@ -3938,7 +3938,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>96.3</v>
+        <v>12.8</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>105511</v>
+        <v>4006</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>62.47</v>
+        <v>106.69</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>105490</v>
+        <v>105236</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>246.9</v>
+        <v>1155.57</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4025,15 +4025,15 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>84530</v>
+        <v>145757</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4041,15 +4041,15 @@
         <v>46281</v>
       </c>
       <c r="H93" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>48.14</v>
+        <v>128.22</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4062,15 +4062,15 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>140516</v>
+        <v>105465</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4078,15 +4078,15 @@
         <v>46281</v>
       </c>
       <c r="H94" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>108.8</v>
+        <v>96.3</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4099,15 +4099,15 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>162989</v>
+        <v>105511</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4115,15 +4115,15 @@
         <v>46281</v>
       </c>
       <c r="H95" t="n">
-        <v>796770</v>
+        <v>789423</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>155.18</v>
+        <v>62.47</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4136,37 +4136,31 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>1031</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H96" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>57.06</v>
+        <v>256.32</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4179,37 +4173,31 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>70696</v>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>2605007</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>105490</v>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H97" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>82.98</v>
+        <v>246.9</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4230,29 +4218,23 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>154430</v>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>NEG02225</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>84530</v>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H98" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>29.46</v>
+        <v>48.14</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4273,29 +4255,23 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>140705</v>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>0000301524</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>140516</v>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H99" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>39.98</v>
+        <v>108.8</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4308,37 +4284,31 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>153194</v>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>0000297125</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="n">
-        <v>46508</v>
-      </c>
+        <v>162989</v>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H100" t="n">
-        <v>789423</v>
+        <v>796770</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>55.4</v>
+        <v>155.18</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4359,29 +4329,29 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>143552</v>
+        <v>161944</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>0000289416</t>
+          <t>2514837</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>46661</v>
+        <v>46813</v>
       </c>
       <c r="G101" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H101" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>23.94</v>
+        <v>57.06</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4394,31 +4364,37 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>141811</v>
-      </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
+        <v>70696</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2605007</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G102" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H102" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>107.64</v>
+        <v>82.98</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4431,31 +4407,37 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>162443</v>
-      </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
+        <v>154430</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>NEG02225</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G103" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H103" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>220.91</v>
+        <v>29.46</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4468,18 +4450,24 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
+        <v>140705</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>0000301524</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G104" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4492,7 +4480,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>482.65</v>
+        <v>39.98</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4505,18 +4493,24 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>2283</v>
-      </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
+        <v>153194</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>46508</v>
+      </c>
       <c r="G105" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4529,7 +4523,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>318.34</v>
+        <v>55.4</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4542,18 +4536,24 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>7226</v>
-      </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G106" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>293.44</v>
+        <v>23.94</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>105228</v>
+        <v>2283</v>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>2753.62</v>
+        <v>424.45</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4624,7 +4624,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>145423</v>
+        <v>141811</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>257.04</v>
+        <v>107.64</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>140716</v>
+        <v>162443</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
@@ -4677,9 +4677,268 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>113.25</v>
+        <v>1546.38</v>
       </c>
       <c r="K109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>142</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>140716</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H110" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>226.5</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>142</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H111" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>1061.83</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>142</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>145691</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H112" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>85.43000000000001</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>142</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>7226</v>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H113" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>293.44</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>142</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>105228</v>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H114" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>2753.62</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>142</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>145423</v>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H115" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>142</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H116" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>552.45</v>
+      </c>
+      <c r="K116" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 12:45:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>140719</v>
+        <v>156557</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>214.71</v>
+        <v>498.25</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8451</v>
+        <v>140719</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>435.41</v>
+        <v>214.71</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>142054</v>
+        <v>8451</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>271.48</v>
+        <v>435.41</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>105481</v>
+        <v>142054</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>973.14</v>
+        <v>271.48</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>143382</v>
+        <v>105481</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>238.04</v>
+        <v>973.14</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>128896</v>
+        <v>143382</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>118.12</v>
+        <v>238.04</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>155062</v>
+        <v>128896</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2311.03</v>
+        <v>118.12</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1600</v>
+        <v>155062</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>121.72</v>
+        <v>2311.03</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>149872</v>
+        <v>1600</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>45.6</v>
+        <v>121.72</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1365,37 +1365,31 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>A09A06326</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>149872</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H25" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>33.04</v>
+        <v>45.6</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1408,31 +1402,37 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>141919</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+        <v>141361</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>A09A06326</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G26" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>30307</v>
+        <v>31305</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>210.43</v>
+        <v>33.04</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>156110</v>
+        <v>141919</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>166.48</v>
+        <v>210.43</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>157509</v>
+        <v>156110</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>145.61</v>
+        <v>166.48</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1519,15 +1519,15 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>162951</v>
+        <v>157509</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1535,15 +1535,15 @@
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>155.18</v>
+        <v>145.61</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1556,37 +1556,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>162951</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>31.51</v>
+        <v>155.18</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1607,29 +1601,29 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>161738</v>
+        <v>140308</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>B26B1405</t>
+          <t>2518727</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46784</v>
+        <v>46722</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>16.79</v>
+        <v>31.51</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1650,29 +1644,29 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>155062</v>
+        <v>161738</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0000293487</t>
+          <t>B26B1405</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>47119</v>
+        <v>46784</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H32" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>63.38</v>
+        <v>16.79</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1693,15 +1687,15 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>140746</v>
+        <v>155062</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0000291396</t>
+          <t>0000293487</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46784</v>
+        <v>47119</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
@@ -1715,7 +1709,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>68.16</v>
+        <v>63.38</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1736,15 +1730,15 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>161127</v>
+        <v>140746</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0000293755</t>
+          <t>0000291396</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46753</v>
+        <v>46784</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46281</v>
@@ -1758,7 +1752,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>21.12</v>
+        <v>68.16</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1779,15 +1773,15 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>145691</v>
+        <v>161127</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0000287662</t>
+          <t>0000293755</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46631</v>
+        <v>46753</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46281</v>
@@ -1801,7 +1795,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>38.72</v>
+        <v>21.12</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1814,18 +1808,24 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>127998</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
+        <v>145691</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0000287662</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>46631</v>
+      </c>
       <c r="G36" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>651.15</v>
+        <v>38.72</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>162453</v>
+        <v>127998</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>151.35</v>
+        <v>651.15</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>146046</v>
+        <v>162453</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>112.87</v>
+        <v>151.35</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>159926</v>
+        <v>146046</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>248.25</v>
+        <v>112.87</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>140745</v>
+        <v>159926</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>1248.4</v>
+        <v>248.25</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>105600</v>
+        <v>140745</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>242.61</v>
+        <v>1248.4</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2036,37 +2036,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H42" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>11.27</v>
+        <v>242.61</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2087,15 +2081,15 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>39233</v>
+        <v>148126</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46905</v>
+        <v>46874</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46281</v>
@@ -2109,7 +2103,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>17.83</v>
+        <v>11.27</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2130,23 +2124,29 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>113875</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G44" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>13.5</v>
+        <v>17.83</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2167,29 +2167,23 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>B26E1180</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>113875</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H45" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8.83</v>
+        <v>13.5</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2210,15 +2204,15 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>141092</v>
+        <v>152321</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>B26E1386</t>
+          <t>B26E1180</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46874</v>
+        <v>46813</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46281</v>
@@ -2232,7 +2226,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>7.29</v>
+        <v>8.83</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2253,15 +2247,15 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>157889</v>
+        <v>141092</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2502015</t>
+          <t>B26E1386</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46844</v>
+        <v>46874</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46281</v>
@@ -2275,7 +2269,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>8.33</v>
+        <v>7.29</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2296,29 +2290,29 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>145423</v>
+        <v>157889</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000292962</t>
+          <t>2502015</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46753</v>
+        <v>46844</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H48" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>58.28</v>
+        <v>8.33</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2339,11 +2333,11 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>157169</v>
+        <v>145423</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>0000292962</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2361,7 +2355,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>23.7</v>
+        <v>58.28</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2382,10 +2376,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G50" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>9.35</v>
+        <v>23.7</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2419,7 +2419,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2448,11 +2448,11 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>271.48</v>
+        <v>12.8</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>66656</v>
+        <v>141180</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>236.76</v>
+        <v>271.48</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>140753</v>
+        <v>66656</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>118.12</v>
+        <v>236.76</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>140718</v>
+        <v>140753</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>427.44</v>
+        <v>118.12</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>143381</v>
+        <v>140718</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>367.36</v>
+        <v>427.44</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>140709</v>
+        <v>143381</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>165.61</v>
+        <v>367.36</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>22098</v>
+        <v>140709</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>62.47</v>
+        <v>165.61</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>46728</v>
+        <v>22098</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>333.04</v>
+        <v>62.47</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>157574</v>
+        <v>46728</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>483.7</v>
+        <v>333.04</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>143553</v>
+        <v>157574</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>424.78</v>
+        <v>483.7</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2818,15 +2818,15 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>163624</v>
+        <v>143553</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2834,15 +2834,15 @@
         <v>46281</v>
       </c>
       <c r="H62" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>104.97</v>
+        <v>424.78</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2855,37 +2855,31 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>163624</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H63" t="n">
-        <v>789825</v>
+        <v>793186</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>67.54000000000001</v>
+        <v>104.97</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2898,31 +2892,37 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>136630</v>
-      </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G64" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H64" t="n">
-        <v>30307</v>
+        <v>789825</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>239.16</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>163047</v>
+        <v>136630</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>226.84</v>
+        <v>239.16</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2980,29 +2980,23 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>0000289599</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>163047</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H66" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>29.12</v>
+        <v>226.84</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3015,18 +3009,24 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>143384</v>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G67" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>653.86</v>
+        <v>29.12</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>140710</v>
+        <v>143384</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>549.87</v>
+        <v>653.86</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>105546</v>
+        <v>140710</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>959.7</v>
+        <v>549.87</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>155959</v>
+        <v>105546</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>310.29</v>
+        <v>959.7</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3163,37 +3163,31 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>155959</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
       <c r="G71" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H71" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>12.86</v>
+        <v>310.29</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3214,23 +3208,29 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G72" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H72" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>103.48</v>
+        <v>12.86</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3243,15 +3243,15 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>84026</v>
+        <v>162584</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
@@ -3259,15 +3259,15 @@
         <v>46281</v>
       </c>
       <c r="H73" t="n">
-        <v>33928</v>
+        <v>793186</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>81.25</v>
+        <v>103.48</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3288,16 +3288,10 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>84026</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3310,7 +3304,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>43.6</v>
+        <v>81.25</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3323,37 +3317,37 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>79510</v>
+        <v>123480</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>2517347</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H75" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>8.84</v>
+        <v>43.6</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3374,15 +3368,15 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>161224</v>
+        <v>79510</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>B26F1555</t>
+          <t>B26C2880</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>46905</v>
+        <v>46844</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>46281</v>
@@ -3396,7 +3390,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>31.97</v>
+        <v>8.84</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3409,31 +3403,37 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>142053</v>
-      </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
+        <v>161224</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>B26F1555</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G77" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H77" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>271.48</v>
+        <v>31.97</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>145623</v>
+        <v>142053</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>208.71</v>
+        <v>271.48</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3491,7 +3491,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>162452</v>
+        <v>145623</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>212.22</v>
+        <v>208.71</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>142886</v>
+        <v>162452</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3544,7 +3544,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>54.88</v>
+        <v>212.22</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1120</v>
+        <v>142886</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>237.8</v>
+        <v>54.88</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3602,7 +3602,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>27723</v>
+        <v>1120</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>385.19</v>
+        <v>237.8</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3631,15 +3631,15 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>113883</v>
+        <v>27723</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3647,15 +3647,15 @@
         <v>46281</v>
       </c>
       <c r="H83" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>13.5</v>
+        <v>385.19</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3668,15 +3668,15 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>158354</v>
+        <v>113883</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3684,15 +3684,15 @@
         <v>46281</v>
       </c>
       <c r="H84" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>198.58</v>
+        <v>13.5</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3705,37 +3705,31 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>7.69</v>
+        <v>198.58</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3756,15 +3750,15 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>122050</v>
+        <v>95842</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2519527</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>46905</v>
+        <v>46753</v>
       </c>
       <c r="G86" s="2" t="n">
         <v>46281</v>
@@ -3778,7 +3772,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>49.61</v>
+        <v>7.69</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3799,15 +3793,15 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>140846</v>
+        <v>122050</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>46813</v>
+        <v>46905</v>
       </c>
       <c r="G87" s="2" t="n">
         <v>46281</v>
@@ -3821,7 +3815,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>22</v>
+        <v>49.61</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3842,15 +3836,15 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>151540</v>
+        <v>140846</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>46569</v>
+        <v>46813</v>
       </c>
       <c r="G88" s="2" t="n">
         <v>46281</v>
@@ -3864,7 +3858,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>12.46</v>
+        <v>22</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3885,23 +3879,29 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>157926</v>
-      </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G89" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H89" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>22.3</v>
+        <v>12.46</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>142054</v>
+        <v>157926</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
@@ -3938,7 +3938,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>12.8</v>
+        <v>22.3</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3951,15 +3951,15 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>4006</v>
+        <v>142054</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>106.69</v>
+        <v>12.8</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>105236</v>
+        <v>4006</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>1155.57</v>
+        <v>106.69</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>145757</v>
+        <v>105236</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>128.22</v>
+        <v>1155.57</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>105465</v>
+        <v>145757</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4086,7 +4086,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>96.3</v>
+        <v>128.22</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>105511</v>
+        <v>105465</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>62.47</v>
+        <v>96.3</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4144,7 +4144,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1031</v>
+        <v>105511</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>256.32</v>
+        <v>62.47</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>105490</v>
+        <v>1031</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>246.9</v>
+        <v>256.32</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4210,15 +4210,15 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>84530</v>
+        <v>105490</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
@@ -4226,15 +4226,15 @@
         <v>46281</v>
       </c>
       <c r="H98" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>48.14</v>
+        <v>246.9</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4255,7 +4255,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>140516</v>
+        <v>84530</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
@@ -4263,15 +4263,15 @@
         <v>46281</v>
       </c>
       <c r="H99" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>108.8</v>
+        <v>48.14</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4284,15 +4284,15 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>162989</v>
+        <v>140516</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
@@ -4300,15 +4300,15 @@
         <v>46281</v>
       </c>
       <c r="H100" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>155.18</v>
+        <v>108.8</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4321,37 +4321,31 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F101" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>162989</v>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H101" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>57.06</v>
+        <v>155.18</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4364,23 +4358,23 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>70696</v>
+        <v>161944</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2605007</t>
+          <t>2514837</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>46844</v>
+        <v>46813</v>
       </c>
       <c r="G102" s="2" t="n">
         <v>46281</v>
@@ -4394,7 +4388,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>82.98</v>
+        <v>57.06</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4407,37 +4401,37 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>154430</v>
+        <v>70696</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>NEG02225</t>
+          <t>2605007</t>
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>46692</v>
+        <v>46844</v>
       </c>
       <c r="G103" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H103" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>29.46</v>
+        <v>82.98</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4458,29 +4452,29 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>140705</v>
+        <v>154430</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>0000301524</t>
+          <t>NEG02225</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H104" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>39.98</v>
+        <v>29.46</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4501,15 +4495,15 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>153194</v>
+        <v>140705</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>0000297125</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>46508</v>
+        <v>46844</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>46281</v>
@@ -4523,7 +4517,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>55.4</v>
+        <v>39.98</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4544,15 +4538,15 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>143552</v>
+        <v>153194</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>0000289416</t>
+          <t>0000297125</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>46661</v>
+        <v>46508</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>46281</v>
@@ -4566,7 +4560,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>23.94</v>
+        <v>55.4</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4579,18 +4573,24 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>2283</v>
-      </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G107" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>424.45</v>
+        <v>23.94</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4624,7 +4624,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>141811</v>
+        <v>2283</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>107.64</v>
+        <v>424.45</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>162443</v>
+        <v>141811</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>1546.38</v>
+        <v>107.64</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -4698,7 +4698,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>140716</v>
+        <v>162443</v>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
@@ -4714,7 +4714,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>226.5</v>
+        <v>1546.38</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>155058</v>
+        <v>140716</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>1061.83</v>
+        <v>226.5</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>145691</v>
+        <v>155058</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -4788,7 +4788,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>85.43000000000001</v>
+        <v>1061.83</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -4809,7 +4809,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>7226</v>
+        <v>145691</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>293.44</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -4846,7 +4846,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>105228</v>
+        <v>7226</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>2753.62</v>
+        <v>293.44</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>145423</v>
+        <v>105228</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>453.76</v>
+        <v>2753.62</v>
       </c>
       <c r="K115" t="n">
         <v>0</v>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>140746</v>
+        <v>145423</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -4936,9 +4936,46 @@
         </is>
       </c>
       <c r="J116" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>142</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H117" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
         <v>552.45</v>
       </c>
-      <c r="K116" t="n">
+      <c r="K117" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:30:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -952,37 +952,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>155058</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0000281593</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>17590</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H14" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>47.66</v>
+        <v>459.65</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1003,10 +997,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4006</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+        <v>155058</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0000281593</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>12.48</v>
+        <v>47.66</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1032,15 +1032,15 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>156557</v>
+        <v>4006</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>498.25</v>
+        <v>12.48</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>140719</v>
+        <v>156557</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>214.71</v>
+        <v>498.25</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8451</v>
+        <v>140719</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>435.41</v>
+        <v>214.71</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>142054</v>
+        <v>8451</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>271.48</v>
+        <v>435.41</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>105481</v>
+        <v>142054</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>973.14</v>
+        <v>271.48</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>143382</v>
+        <v>105481</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>238.04</v>
+        <v>973.14</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>128896</v>
+        <v>143382</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>118.12</v>
+        <v>238.04</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>155062</v>
+        <v>128896</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2311.03</v>
+        <v>118.12</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1600</v>
+        <v>155062</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>121.72</v>
+        <v>2311.03</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>149872</v>
+        <v>1600</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>45.6</v>
+        <v>121.72</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1402,37 +1402,31 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>A09A06326</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>149872</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H26" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>33.04</v>
+        <v>45.6</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1445,31 +1439,37 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>141919</v>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+        <v>141361</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>A09A06326</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G27" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H27" t="n">
-        <v>30307</v>
+        <v>31305</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>210.43</v>
+        <v>33.04</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>156110</v>
+        <v>141919</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>166.48</v>
+        <v>210.43</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>157509</v>
+        <v>156110</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>145.61</v>
+        <v>166.48</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1556,15 +1556,15 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>162951</v>
+        <v>157509</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
@@ -1572,15 +1572,15 @@
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>155.18</v>
+        <v>145.61</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1593,37 +1593,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>162951</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>31.51</v>
+        <v>155.18</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1644,29 +1638,29 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>161738</v>
+        <v>140308</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>B26B1405</t>
+          <t>2518727</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46784</v>
+        <v>46722</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H32" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>16.79</v>
+        <v>31.51</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1687,29 +1681,29 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>155062</v>
+        <v>161738</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0000293487</t>
+          <t>B26B1405</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>47119</v>
+        <v>46784</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>63.38</v>
+        <v>16.79</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1730,15 +1724,15 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>140746</v>
+        <v>155062</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0000291396</t>
+          <t>0000293487</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46784</v>
+        <v>47119</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46281</v>
@@ -1752,7 +1746,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>68.16</v>
+        <v>63.38</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1773,15 +1767,15 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>161127</v>
+        <v>140746</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0000293755</t>
+          <t>0000291396</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46753</v>
+        <v>46784</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46281</v>
@@ -1795,7 +1789,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>21.12</v>
+        <v>68.16</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1816,15 +1810,15 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>145691</v>
+        <v>161127</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0000287662</t>
+          <t>0000293755</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46631</v>
+        <v>46753</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46281</v>
@@ -1838,7 +1832,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>38.72</v>
+        <v>21.12</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1851,18 +1845,24 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>127998</v>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
+        <v>145691</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0000287662</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>46631</v>
+      </c>
       <c r="G37" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>651.15</v>
+        <v>38.72</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>162453</v>
+        <v>127998</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>151.35</v>
+        <v>651.15</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>146046</v>
+        <v>162453</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>112.87</v>
+        <v>151.35</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>159926</v>
+        <v>146046</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>248.25</v>
+        <v>112.87</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>140745</v>
+        <v>159926</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>1248.4</v>
+        <v>248.25</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>105600</v>
+        <v>140745</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>242.61</v>
+        <v>1248.4</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2073,37 +2073,31 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>148126</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>A90B00326</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H43" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>11.27</v>
+        <v>242.61</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2124,15 +2118,15 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>39233</v>
+        <v>148126</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46905</v>
+        <v>46874</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46281</v>
@@ -2146,7 +2140,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>17.83</v>
+        <v>11.27</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2167,23 +2161,29 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>113875</v>
-      </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G45" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H45" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>13.5</v>
+        <v>17.83</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2204,29 +2204,23 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>B26E1180</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>113875</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H46" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>8.83</v>
+        <v>13.5</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2247,15 +2241,15 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>141092</v>
+        <v>152321</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>B26E1386</t>
+          <t>B26E1180</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46874</v>
+        <v>46813</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46281</v>
@@ -2269,7 +2263,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>7.29</v>
+        <v>8.83</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2290,15 +2284,15 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>157889</v>
+        <v>141092</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2502015</t>
+          <t>B26E1386</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46844</v>
+        <v>46874</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46281</v>
@@ -2312,7 +2306,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>8.33</v>
+        <v>7.29</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2333,29 +2327,29 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>145423</v>
+        <v>157889</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0000292962</t>
+          <t>2502015</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46753</v>
+        <v>46844</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H49" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>58.28</v>
+        <v>8.33</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2376,11 +2370,11 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>157169</v>
+        <v>145423</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>0000292962</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -2398,7 +2392,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>23.7</v>
+        <v>58.28</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2419,10 +2413,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G51" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2435,7 +2435,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>9.35</v>
+        <v>23.7</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2485,11 +2485,11 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>271.48</v>
+        <v>12.8</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>66656</v>
+        <v>141180</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>236.76</v>
+        <v>271.48</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>140753</v>
+        <v>66656</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>118.12</v>
+        <v>236.76</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>140718</v>
+        <v>140753</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>427.44</v>
+        <v>118.12</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>143381</v>
+        <v>140718</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>367.36</v>
+        <v>427.44</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>140709</v>
+        <v>143381</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>165.61</v>
+        <v>367.36</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>22098</v>
+        <v>140709</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>62.47</v>
+        <v>165.61</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>46728</v>
+        <v>22098</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>333.04</v>
+        <v>62.47</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>157574</v>
+        <v>46728</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>483.7</v>
+        <v>333.04</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2826,7 +2826,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>143553</v>
+        <v>157574</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>424.78</v>
+        <v>483.7</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2855,15 +2855,15 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>163624</v>
+        <v>143553</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -2871,15 +2871,15 @@
         <v>46281</v>
       </c>
       <c r="H63" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>104.97</v>
+        <v>424.78</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2892,37 +2892,31 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>163624</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H64" t="n">
-        <v>789825</v>
+        <v>793186</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>67.54000000000001</v>
+        <v>104.97</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2935,31 +2929,37 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>136630</v>
-      </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G65" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H65" t="n">
-        <v>30307</v>
+        <v>789825</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>239.16</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>163047</v>
+        <v>136630</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>226.84</v>
+        <v>239.16</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3017,29 +3017,23 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>0000289599</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>163047</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H67" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>29.12</v>
+        <v>226.84</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3052,18 +3046,24 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>143384</v>
-      </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G68" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>653.86</v>
+        <v>29.12</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>140710</v>
+        <v>143384</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>549.87</v>
+        <v>653.86</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>105546</v>
+        <v>140710</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>959.7</v>
+        <v>549.87</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>155959</v>
+        <v>105546</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>310.29</v>
+        <v>959.7</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3200,37 +3200,31 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>155959</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H72" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>12.86</v>
+        <v>310.29</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3251,23 +3245,29 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G73" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H73" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>103.48</v>
+        <v>12.86</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3280,15 +3280,15 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>84026</v>
+        <v>162584</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
@@ -3296,15 +3296,15 @@
         <v>46281</v>
       </c>
       <c r="H74" t="n">
-        <v>33928</v>
+        <v>793186</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>81.25</v>
+        <v>103.48</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3325,16 +3325,10 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>84026</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
       <c r="G75" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3347,7 +3341,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>43.6</v>
+        <v>81.25</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3360,37 +3354,37 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>79510</v>
+        <v>123480</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>2517347</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H76" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>8.84</v>
+        <v>43.6</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3411,15 +3405,15 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>161224</v>
+        <v>79510</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>B26F1555</t>
+          <t>B26C2880</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>46905</v>
+        <v>46844</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>46281</v>
@@ -3433,7 +3427,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>31.97</v>
+        <v>8.84</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3446,31 +3440,37 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>142053</v>
-      </c>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
+        <v>161224</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>B26F1555</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G78" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H78" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>271.48</v>
+        <v>31.97</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3491,7 +3491,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>145623</v>
+        <v>142053</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>208.71</v>
+        <v>271.48</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>162452</v>
+        <v>145623</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3544,7 +3544,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>212.22</v>
+        <v>208.71</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>142886</v>
+        <v>162452</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>54.88</v>
+        <v>212.22</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3602,7 +3602,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1120</v>
+        <v>142886</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>237.8</v>
+        <v>54.88</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>27723</v>
+        <v>1120</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>385.19</v>
+        <v>237.8</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3668,15 +3668,15 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>113883</v>
+        <v>27723</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3684,15 +3684,15 @@
         <v>46281</v>
       </c>
       <c r="H84" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>13.5</v>
+        <v>385.19</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3705,15 +3705,15 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>158354</v>
+        <v>113883</v>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
@@ -3721,15 +3721,15 @@
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>198.58</v>
+        <v>13.5</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3742,37 +3742,31 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
       <c r="G86" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H86" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>7.69</v>
+        <v>198.58</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3793,15 +3787,15 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>122050</v>
+        <v>95842</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2519527</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>46905</v>
+        <v>46753</v>
       </c>
       <c r="G87" s="2" t="n">
         <v>46281</v>
@@ -3815,7 +3809,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>49.61</v>
+        <v>7.69</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3836,15 +3830,15 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>140846</v>
+        <v>122050</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>46813</v>
+        <v>46905</v>
       </c>
       <c r="G88" s="2" t="n">
         <v>46281</v>
@@ -3858,7 +3852,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>22</v>
+        <v>49.61</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3879,15 +3873,15 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>151540</v>
+        <v>140846</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>46569</v>
+        <v>46813</v>
       </c>
       <c r="G89" s="2" t="n">
         <v>46281</v>
@@ -3901,7 +3895,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>12.46</v>
+        <v>22</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3922,23 +3916,29 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>157926</v>
-      </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G90" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H90" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>22.3</v>
+        <v>12.46</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>142054</v>
+        <v>157926</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>12.8</v>
+        <v>22.3</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3988,15 +3988,15 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>4006</v>
+        <v>142054</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>106.69</v>
+        <v>12.8</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>105236</v>
+        <v>4006</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>1155.57</v>
+        <v>106.69</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>145757</v>
+        <v>105236</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4086,7 +4086,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>128.22</v>
+        <v>1155.57</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>105465</v>
+        <v>145757</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>96.3</v>
+        <v>128.22</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4144,7 +4144,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>105511</v>
+        <v>105465</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>62.47</v>
+        <v>96.3</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>1031</v>
+        <v>105511</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>256.32</v>
+        <v>62.47</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4218,7 +4218,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>105490</v>
+        <v>1031</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>246.9</v>
+        <v>256.32</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4247,15 +4247,15 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>84530</v>
+        <v>105490</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
@@ -4263,15 +4263,15 @@
         <v>46281</v>
       </c>
       <c r="H99" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>48.14</v>
+        <v>246.9</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>140516</v>
+        <v>84530</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
@@ -4300,15 +4300,15 @@
         <v>46281</v>
       </c>
       <c r="H100" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>108.8</v>
+        <v>48.14</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4321,15 +4321,15 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>162989</v>
+        <v>140516</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
@@ -4337,15 +4337,15 @@
         <v>46281</v>
       </c>
       <c r="H101" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>155.18</v>
+        <v>108.8</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4358,37 +4358,31 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>162989</v>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H102" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>57.06</v>
+        <v>155.18</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4401,23 +4395,23 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>70696</v>
+        <v>161944</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2605007</t>
+          <t>2514837</t>
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>46844</v>
+        <v>46813</v>
       </c>
       <c r="G103" s="2" t="n">
         <v>46281</v>
@@ -4431,7 +4425,7 @@
         </is>
       </c>
       <c r="J103" t="n">
-        <v>82.98</v>
+        <v>57.06</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4444,37 +4438,37 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>154430</v>
+        <v>70696</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>NEG02225</t>
+          <t>2605007</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>46692</v>
+        <v>46844</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H104" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>29.46</v>
+        <v>82.98</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4495,29 +4489,29 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>140705</v>
+        <v>154430</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>0000301524</t>
+          <t>NEG02225</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H105" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>39.98</v>
+        <v>29.46</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4538,15 +4532,15 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>153194</v>
+        <v>140705</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>0000297125</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>46508</v>
+        <v>46844</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>46281</v>
@@ -4560,7 +4554,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>55.4</v>
+        <v>39.98</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4581,15 +4575,15 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>143552</v>
+        <v>153194</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>0000289416</t>
+          <t>0000297125</t>
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>46661</v>
+        <v>46508</v>
       </c>
       <c r="G107" s="2" t="n">
         <v>46281</v>
@@ -4603,7 +4597,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>23.94</v>
+        <v>55.4</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4616,18 +4610,24 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>2283</v>
-      </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G108" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>424.45</v>
+        <v>23.94</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>141811</v>
+        <v>2283</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>107.64</v>
+        <v>424.45</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -4698,7 +4698,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>162443</v>
+        <v>141811</v>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
@@ -4714,7 +4714,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>1546.38</v>
+        <v>107.64</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>140716</v>
+        <v>162443</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>226.5</v>
+        <v>1546.38</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>155058</v>
+        <v>140716</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -4788,7 +4788,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>1061.83</v>
+        <v>226.5</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -4809,7 +4809,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>145691</v>
+        <v>155058</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>85.43000000000001</v>
+        <v>1061.83</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -4846,7 +4846,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>7226</v>
+        <v>145691</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>293.44</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>105228</v>
+        <v>7226</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>2753.62</v>
+        <v>293.44</v>
       </c>
       <c r="K115" t="n">
         <v>0</v>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>145423</v>
+        <v>105228</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -4936,7 +4936,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>453.76</v>
+        <v>2753.62</v>
       </c>
       <c r="K116" t="n">
         <v>0</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>140746</v>
+        <v>145423</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
@@ -4973,9 +4973,46 @@
         </is>
       </c>
       <c r="J117" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>142</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H118" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
         <v>552.45</v>
       </c>
-      <c r="K117" t="n">
+      <c r="K118" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:00:03
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2233,37 +2233,31 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>B26E1180</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>146828</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>8.83</v>
+        <v>15.43</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2284,15 +2278,15 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>141092</v>
+        <v>152321</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>B26E1386</t>
+          <t>B26E1180</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46874</v>
+        <v>46813</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46281</v>
@@ -2306,7 +2300,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>7.29</v>
+        <v>8.83</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2327,15 +2321,15 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>157889</v>
+        <v>141092</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2502015</t>
+          <t>B26E1386</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46844</v>
+        <v>46874</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46281</v>
@@ -2349,7 +2343,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>8.33</v>
+        <v>7.29</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2370,29 +2364,29 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>145423</v>
+        <v>157889</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0000292962</t>
+          <t>2502015</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46753</v>
+        <v>46844</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H50" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>58.28</v>
+        <v>8.33</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2413,11 +2407,11 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>157169</v>
+        <v>145423</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>0000292962</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -2435,7 +2429,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>23.7</v>
+        <v>58.28</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2456,10 +2450,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G52" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>9.35</v>
+        <v>23.7</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>141180</v>
+        <v>134701</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>12.8</v>
+        <v>9.35</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2522,11 +2522,11 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2546,7 +2546,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>271.48</v>
+        <v>12.8</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>66656</v>
+        <v>141180</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>236.76</v>
+        <v>271.48</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>140753</v>
+        <v>66656</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>118.12</v>
+        <v>236.76</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>140718</v>
+        <v>140753</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>427.44</v>
+        <v>118.12</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>143381</v>
+        <v>140718</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>367.36</v>
+        <v>427.44</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>140709</v>
+        <v>143381</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>165.61</v>
+        <v>367.36</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>22098</v>
+        <v>140709</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>62.47</v>
+        <v>165.61</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>46728</v>
+        <v>22098</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>333.04</v>
+        <v>62.47</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2826,7 +2826,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>157574</v>
+        <v>46728</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>483.7</v>
+        <v>333.04</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>143553</v>
+        <v>157574</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>424.78</v>
+        <v>483.7</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2892,15 +2892,15 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>163624</v>
+        <v>143553</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -2908,15 +2908,15 @@
         <v>46281</v>
       </c>
       <c r="H64" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>104.97</v>
+        <v>424.78</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2929,37 +2929,31 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>163624</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H65" t="n">
-        <v>789825</v>
+        <v>793186</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>67.54000000000001</v>
+        <v>104.97</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2972,31 +2966,37 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>136630</v>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G66" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H66" t="n">
-        <v>30307</v>
+        <v>789825</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>239.16</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>163047</v>
+        <v>136630</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3033,7 +3033,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>226.84</v>
+        <v>239.16</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3054,29 +3054,23 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>0000289599</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>163047</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H68" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>29.12</v>
+        <v>226.84</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3089,18 +3083,24 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>143384</v>
-      </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
+        <v>140738</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>0000289599</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G69" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>653.86</v>
+        <v>29.12</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>140710</v>
+        <v>143384</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>549.87</v>
+        <v>653.86</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>105546</v>
+        <v>140710</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>959.7</v>
+        <v>549.87</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>155959</v>
+        <v>105546</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -3224,7 +3224,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>310.29</v>
+        <v>959.7</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3237,37 +3237,31 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>155959</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H73" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>12.86</v>
+        <v>310.29</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3288,23 +3282,29 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G74" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H74" t="n">
-        <v>793186</v>
+        <v>31305</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>103.48</v>
+        <v>12.86</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3317,15 +3317,15 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>84026</v>
+        <v>162584</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -3333,15 +3333,15 @@
         <v>46281</v>
       </c>
       <c r="H75" t="n">
-        <v>33928</v>
+        <v>793186</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>81.25</v>
+        <v>103.48</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3362,16 +3362,10 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>84026</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3384,7 +3378,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>43.6</v>
+        <v>81.25</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3397,37 +3391,37 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>79510</v>
+        <v>123480</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>2517347</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H77" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>8.84</v>
+        <v>43.6</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3448,15 +3442,15 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>161224</v>
+        <v>79510</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>B26F1555</t>
+          <t>B26C2880</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>46905</v>
+        <v>46844</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>46281</v>
@@ -3470,7 +3464,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>31.97</v>
+        <v>8.84</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3483,31 +3477,37 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>142053</v>
-      </c>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
+        <v>161224</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>B26F1555</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G79" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H79" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>271.48</v>
+        <v>31.97</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>145623</v>
+        <v>142053</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3544,7 +3544,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>208.71</v>
+        <v>271.48</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>162452</v>
+        <v>145623</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>212.22</v>
+        <v>208.71</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3602,7 +3602,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>142886</v>
+        <v>162452</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>54.88</v>
+        <v>212.22</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1120</v>
+        <v>142886</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>237.8</v>
+        <v>54.88</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3676,7 +3676,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>27723</v>
+        <v>1120</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>385.19</v>
+        <v>237.8</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3705,15 +3705,15 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>113883</v>
+        <v>27723</v>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
@@ -3721,15 +3721,15 @@
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>13.5</v>
+        <v>385.19</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3742,15 +3742,15 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>158354</v>
+        <v>113883</v>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
@@ -3758,15 +3758,15 @@
         <v>46281</v>
       </c>
       <c r="H86" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>198.58</v>
+        <v>13.5</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3779,37 +3779,31 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>95842</v>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>2519527</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>158354</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H87" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>7.69</v>
+        <v>198.58</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3830,15 +3824,15 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>122050</v>
+        <v>95842</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2608233</t>
+          <t>2519527</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>46905</v>
+        <v>46753</v>
       </c>
       <c r="G88" s="2" t="n">
         <v>46281</v>
@@ -3852,7 +3846,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>49.61</v>
+        <v>7.69</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3873,15 +3867,15 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>140846</v>
+        <v>122050</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2603107</t>
+          <t>2608233</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>46813</v>
+        <v>46905</v>
       </c>
       <c r="G89" s="2" t="n">
         <v>46281</v>
@@ -3895,7 +3889,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>22</v>
+        <v>49.61</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3916,15 +3910,15 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>151540</v>
+        <v>140846</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>20012026</t>
+          <t>2603107</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>46569</v>
+        <v>46813</v>
       </c>
       <c r="G90" s="2" t="n">
         <v>46281</v>
@@ -3938,7 +3932,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>12.46</v>
+        <v>22</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3959,23 +3953,29 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>157926</v>
-      </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G91" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H91" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>22.3</v>
+        <v>12.46</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3996,7 +3996,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>142054</v>
+        <v>157926</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>12.8</v>
+        <v>22.3</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4025,15 +4025,15 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>4006</v>
+        <v>142054</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>106.69</v>
+        <v>12.8</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>105236</v>
+        <v>4006</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4086,7 +4086,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>1155.57</v>
+        <v>106.69</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>145757</v>
+        <v>105236</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>128.22</v>
+        <v>1155.57</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4144,7 +4144,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>105465</v>
+        <v>145757</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>96.3</v>
+        <v>128.22</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>105511</v>
+        <v>105465</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>62.47</v>
+        <v>96.3</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4218,7 +4218,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1031</v>
+        <v>105511</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>256.32</v>
+        <v>62.47</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4255,7 +4255,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>105490</v>
+        <v>1031</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>246.9</v>
+        <v>256.32</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4284,15 +4284,15 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>84530</v>
+        <v>105490</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
@@ -4300,15 +4300,15 @@
         <v>46281</v>
       </c>
       <c r="H100" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>48.14</v>
+        <v>246.9</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4329,7 +4329,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>140516</v>
+        <v>84530</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
@@ -4337,15 +4337,15 @@
         <v>46281</v>
       </c>
       <c r="H101" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>108.8</v>
+        <v>48.14</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4358,15 +4358,15 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>162989</v>
+        <v>140516</v>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
@@ -4374,15 +4374,15 @@
         <v>46281</v>
       </c>
       <c r="H102" t="n">
-        <v>796770</v>
+        <v>30307</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>155.18</v>
+        <v>108.8</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4395,37 +4395,31 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>162989</v>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H103" t="n">
-        <v>33928</v>
+        <v>796770</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>57.06</v>
+        <v>155.18</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4438,23 +4432,23 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>70696</v>
+        <v>161944</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2605007</t>
+          <t>2514837</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>46844</v>
+        <v>46813</v>
       </c>
       <c r="G104" s="2" t="n">
         <v>46281</v>
@@ -4468,7 +4462,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>82.98</v>
+        <v>57.06</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4481,37 +4475,37 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>154430</v>
+        <v>70696</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>NEG02225</t>
+          <t>2605007</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>46692</v>
+        <v>46844</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H105" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>29.46</v>
+        <v>82.98</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4532,29 +4526,29 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>140705</v>
+        <v>154430</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>0000301524</t>
+          <t>NEG02225</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>46844</v>
+        <v>46692</v>
       </c>
       <c r="G106" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H106" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>39.98</v>
+        <v>29.46</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4567,37 +4561,31 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>153194</v>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>0000297125</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="n">
-        <v>46508</v>
-      </c>
+        <v>79367</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H107" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>55.4</v>
+        <v>31.15</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4618,15 +4606,15 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>143552</v>
+        <v>140705</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>0000289416</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>46661</v>
+        <v>46844</v>
       </c>
       <c r="G108" s="2" t="n">
         <v>46281</v>
@@ -4640,7 +4628,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>23.94</v>
+        <v>39.98</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4653,18 +4641,24 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>2283</v>
-      </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
+        <v>153194</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>46508</v>
+      </c>
       <c r="G109" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4677,7 +4671,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>424.45</v>
+        <v>55.4</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -4690,18 +4684,24 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>141811</v>
-      </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G110" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4714,7 +4714,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>107.64</v>
+        <v>23.94</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>162443</v>
+        <v>2283</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>1546.38</v>
+        <v>424.45</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>140716</v>
+        <v>141811</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -4788,7 +4788,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>226.5</v>
+        <v>107.64</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -4809,7 +4809,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>155058</v>
+        <v>162443</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>1061.83</v>
+        <v>1546.38</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -4846,7 +4846,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>145691</v>
+        <v>140716</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>85.43000000000001</v>
+        <v>226.5</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>7226</v>
+        <v>155058</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>293.44</v>
+        <v>1061.83</v>
       </c>
       <c r="K115" t="n">
         <v>0</v>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>105228</v>
+        <v>145691</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -4936,7 +4936,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>2753.62</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="K116" t="n">
         <v>0</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>145423</v>
+        <v>7226</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
@@ -4973,7 +4973,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>453.76</v>
+        <v>293.44</v>
       </c>
       <c r="K117" t="n">
         <v>0</v>
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>140746</v>
+        <v>105228</v>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
@@ -5010,9 +5010,83 @@
         </is>
       </c>
       <c r="J118" t="n">
+        <v>2753.62</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>142</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>145423</v>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H119" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>142</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H120" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
         <v>552.45</v>
       </c>
-      <c r="K118" t="n">
+      <c r="K120" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:30:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K120"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>127998</v>
+        <v>140745</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>651.15</v>
+        <v>1456.47</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>162453</v>
+        <v>127998</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>151.35</v>
+        <v>895.33</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1970,7 +1970,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>146046</v>
+        <v>162453</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>112.87</v>
+        <v>151.35</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>159926</v>
+        <v>146046</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>248.25</v>
+        <v>112.87</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>140745</v>
+        <v>159926</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1248.4</v>
+        <v>248.25</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>236.76</v>
+        <v>285.74</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>142886</v>
+        <v>1120</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>54.88</v>
+        <v>356.7</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3676,7 +3676,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1120</v>
+        <v>142886</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>237.8</v>
+        <v>54.88</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1155.57</v>
+        <v>1540.76</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4598,37 +4598,31 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>140705</v>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>0000301524</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>79375</v>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H108" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J108" t="n">
-        <v>39.98</v>
+        <v>153.69</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4649,15 +4643,15 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>153194</v>
+        <v>140705</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>0000297125</t>
+          <t>0000301524</t>
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>46508</v>
+        <v>46844</v>
       </c>
       <c r="G109" s="2" t="n">
         <v>46281</v>
@@ -4671,7 +4665,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>55.4</v>
+        <v>39.98</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -4692,15 +4686,15 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>143552</v>
+        <v>153194</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>0000289416</t>
+          <t>0000297125</t>
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>46661</v>
+        <v>46508</v>
       </c>
       <c r="G110" s="2" t="n">
         <v>46281</v>
@@ -4714,7 +4708,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>23.94</v>
+        <v>55.4</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -4727,18 +4721,24 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>2283</v>
-      </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G111" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="J111" t="n">
-        <v>424.45</v>
+        <v>23.94</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>141811</v>
+        <v>2283</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -4788,7 +4788,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>107.64</v>
+        <v>424.45</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -4809,7 +4809,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>162443</v>
+        <v>141811</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>1546.38</v>
+        <v>107.64</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -4846,7 +4846,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>140716</v>
+        <v>162443</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>226.5</v>
+        <v>1546.38</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>155058</v>
+        <v>140716</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
@@ -4899,7 +4899,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>1061.83</v>
+        <v>226.5</v>
       </c>
       <c r="K115" t="n">
         <v>0</v>
@@ -4920,7 +4920,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>145691</v>
+        <v>155058</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -4936,7 +4936,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>85.43000000000001</v>
+        <v>1061.83</v>
       </c>
       <c r="K116" t="n">
         <v>0</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>7226</v>
+        <v>145691</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
@@ -4973,7 +4973,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>293.44</v>
+        <v>85.43000000000001</v>
       </c>
       <c r="K117" t="n">
         <v>0</v>
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>105228</v>
+        <v>7226</v>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
@@ -5010,7 +5010,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>2753.62</v>
+        <v>293.44</v>
       </c>
       <c r="K118" t="n">
         <v>0</v>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>145423</v>
+        <v>105228</v>
       </c>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr"/>
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>453.76</v>
+        <v>2753.62</v>
       </c>
       <c r="K119" t="n">
         <v>0</v>
@@ -5068,7 +5068,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>140746</v>
+        <v>145423</v>
       </c>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
@@ -5084,9 +5084,46 @@
         </is>
       </c>
       <c r="J120" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>142</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H121" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
         <v>552.45</v>
       </c>
-      <c r="K120" t="n">
+      <c r="K121" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:00:02
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -866,37 +866,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>98221</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>B25H1859</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>46600</v>
-      </c>
+        <v>145700</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H12" t="n">
-        <v>47252</v>
+        <v>789603</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>SOFTYS BRASIL LTDA</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7.35</v>
+        <v>225.96</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -909,37 +903,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>144460</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>B26E0774</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>163624</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H13" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>6.56</v>
+        <v>703.92</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -952,18 +940,24 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>17590</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+        <v>98221</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B25H1859</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>46600</v>
+      </c>
       <c r="G14" s="2" t="n">
         <v>46281</v>
       </c>
@@ -976,7 +970,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>459.65</v>
+        <v>7.35</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -997,29 +991,29 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>155058</v>
+        <v>144460</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0000281593</t>
+          <t>B26E0774</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46569</v>
+        <v>46874</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H15" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>47.66</v>
+        <v>6.56</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1032,15 +1026,15 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4006</v>
+        <v>17590</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
@@ -1048,15 +1042,15 @@
         <v>46281</v>
       </c>
       <c r="H16" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>12.48</v>
+        <v>459.65</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1069,15 +1063,15 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>156557</v>
+        <v>139212</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -1085,15 +1079,15 @@
         <v>46281</v>
       </c>
       <c r="H17" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>498.25</v>
+        <v>83.67</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1106,18 +1100,24 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>140719</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+        <v>155058</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0000281593</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G18" s="2" t="n">
         <v>46281</v>
       </c>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>214.71</v>
+        <v>47.66</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1143,15 +1143,15 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8451</v>
+        <v>4006</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>435.41</v>
+        <v>12.48</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>142054</v>
+        <v>156557</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>271.48</v>
+        <v>498.25</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>105481</v>
+        <v>140719</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>973.14</v>
+        <v>214.71</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>143382</v>
+        <v>8451</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>238.04</v>
+        <v>435.41</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>128896</v>
+        <v>142054</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>118.12</v>
+        <v>271.48</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>155062</v>
+        <v>105481</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>2311.03</v>
+        <v>973.14</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1600</v>
+        <v>143382</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>121.72</v>
+        <v>238.04</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>149872</v>
+        <v>128896</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>45.6</v>
+        <v>118.12</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1439,37 +1439,31 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>141361</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>A09A06326</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>155062</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H27" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>33.04</v>
+        <v>2311.03</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1482,15 +1476,15 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>141919</v>
+        <v>1600</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
@@ -1498,15 +1492,15 @@
         <v>46281</v>
       </c>
       <c r="H28" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>210.43</v>
+        <v>121.72</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1519,15 +1513,15 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>156110</v>
+        <v>149872</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
@@ -1535,15 +1529,15 @@
         <v>46281</v>
       </c>
       <c r="H29" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>166.48</v>
+        <v>45.6</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1556,31 +1550,37 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>157509</v>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+        <v>141361</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>A09A06326</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G30" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H30" t="n">
-        <v>30307</v>
+        <v>31305</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>145.61</v>
+        <v>33.04</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1601,7 +1601,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>162951</v>
+        <v>144229</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
@@ -1609,15 +1609,15 @@
         <v>46281</v>
       </c>
       <c r="H31" t="n">
-        <v>796770</v>
+        <v>789603</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>SOFTYS BRASIL LTDA</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>155.18</v>
+        <v>188.94</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1630,37 +1630,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>140308</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2518727</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>46722</v>
-      </c>
+        <v>151453</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H32" t="n">
-        <v>33928</v>
+        <v>789603</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>SOFTYS BRASIL LTDA</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>31.51</v>
+        <v>677.87</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1673,37 +1667,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>161738</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>B26B1405</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>46784</v>
-      </c>
+        <v>162584</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H33" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>16.79</v>
+        <v>163.98</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1716,37 +1704,31 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>155062</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>0000293487</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>47119</v>
-      </c>
+        <v>86690</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H34" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>63.38</v>
+        <v>427.92</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1767,29 +1749,23 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>140746</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>0000291396</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>46784</v>
-      </c>
+        <v>141919</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H35" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>68.16</v>
+        <v>210.43</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1810,29 +1786,23 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>161127</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>0000293755</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>156110</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>21.12</v>
+        <v>166.48</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1853,29 +1823,23 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>145691</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>0000287662</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="n">
-        <v>46631</v>
-      </c>
+        <v>157509</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H37" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>38.72</v>
+        <v>145.61</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -1888,15 +1852,15 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>140745</v>
+        <v>162951</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
@@ -1904,15 +1868,15 @@
         <v>46281</v>
       </c>
       <c r="H38" t="n">
-        <v>789423</v>
+        <v>796770</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>1456.47</v>
+        <v>155.18</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1925,31 +1889,37 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>127998</v>
-      </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
+        <v>140308</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2518727</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>46722</v>
+      </c>
       <c r="G39" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H39" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>895.33</v>
+        <v>31.51</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -1962,31 +1932,37 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>162453</v>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
+        <v>161738</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>B26B1405</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>46784</v>
+      </c>
       <c r="G40" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H40" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>151.35</v>
+        <v>16.79</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -1999,15 +1975,15 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>146046</v>
+        <v>111589</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
@@ -2015,15 +1991,15 @@
         <v>46281</v>
       </c>
       <c r="H41" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>112.87</v>
+        <v>27.44</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2036,18 +2012,24 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>159926</v>
-      </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+        <v>155062</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0000293487</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>47119</v>
+      </c>
       <c r="G42" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2060,7 +2042,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>248.25</v>
+        <v>63.38</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2073,18 +2055,24 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>105600</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
+        <v>140746</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0000291396</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46784</v>
+      </c>
       <c r="G43" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2097,7 +2085,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>242.61</v>
+        <v>68.16</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2118,29 +2106,29 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>148126</v>
+        <v>161127</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>A90B00326</t>
+          <t>0000293755</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46874</v>
+        <v>46753</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H44" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>11.27</v>
+        <v>21.12</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2161,29 +2149,29 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>39233</v>
+        <v>145691</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2606104</t>
+          <t>0000287662</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46905</v>
+        <v>46631</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H45" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>17.83</v>
+        <v>38.72</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2196,15 +2184,15 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>113875</v>
+        <v>140745</v>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
@@ -2212,15 +2200,15 @@
         <v>46281</v>
       </c>
       <c r="H46" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>13.5</v>
+        <v>1456.47</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2233,15 +2221,15 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>146828</v>
+        <v>127998</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
@@ -2249,15 +2237,15 @@
         <v>46281</v>
       </c>
       <c r="H47" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>15.43</v>
+        <v>895.33</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2270,37 +2258,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>152321</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>B26E1180</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>162453</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H48" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>8.83</v>
+        <v>151.35</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2313,37 +2295,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>141092</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>B26E1386</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>46874</v>
-      </c>
+        <v>146046</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H49" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>7.29</v>
+        <v>112.87</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2356,37 +2332,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>157889</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2502015</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>159926</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H50" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>8.33</v>
+        <v>248.25</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2399,24 +2369,18 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>145423</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>0000292962</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2429,7 +2393,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>58.28</v>
+        <v>242.61</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2450,29 +2414,29 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>157169</v>
+        <v>148126</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0000294775</t>
+          <t>A90B00326</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46753</v>
+        <v>46874</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H52" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>23.7</v>
+        <v>11.27</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2493,23 +2457,29 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
+        <v>39233</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2606104</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G53" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H53" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>9.35</v>
+        <v>17.83</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -2522,15 +2492,15 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>141180</v>
+        <v>159899</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
@@ -2538,15 +2508,15 @@
         <v>46281</v>
       </c>
       <c r="H54" t="n">
-        <v>789423</v>
+        <v>789603</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>SOFTYS BRASIL LTDA</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>12.8</v>
+        <v>127.74</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -2559,15 +2529,15 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>141180</v>
+        <v>113875</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -2575,15 +2545,15 @@
         <v>46281</v>
       </c>
       <c r="H55" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>271.48</v>
+        <v>13.5</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -2596,15 +2566,15 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>66656</v>
+        <v>146828</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
@@ -2612,15 +2582,15 @@
         <v>46281</v>
       </c>
       <c r="H56" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>285.74</v>
+        <v>15.43</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -2633,31 +2603,37 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>140753</v>
-      </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+        <v>152321</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>B26E1180</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G57" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H57" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>118.12</v>
+        <v>8.83</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -2670,31 +2646,37 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>140718</v>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+        <v>141092</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>B26E1386</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>46874</v>
+      </c>
       <c r="G58" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H58" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>427.44</v>
+        <v>7.29</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -2707,31 +2689,37 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>143381</v>
-      </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
+        <v>157889</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2502015</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G59" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H59" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>367.36</v>
+        <v>8.33</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -2744,18 +2732,24 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>140709</v>
-      </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
+        <v>145423</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0000292962</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G60" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2768,7 +2762,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>165.61</v>
+        <v>58.28</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -2781,18 +2775,24 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>22098</v>
-      </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G61" s="2" t="n">
         <v>46281</v>
       </c>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>62.47</v>
+        <v>23.7</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -2818,15 +2818,15 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>46728</v>
+        <v>134701</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>333.04</v>
+        <v>9.35</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -2855,15 +2855,15 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>157574</v>
+        <v>141180</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>483.7</v>
+        <v>12.8</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -2900,7 +2900,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>143553</v>
+        <v>141180</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
@@ -2916,7 +2916,7 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>424.78</v>
+        <v>271.48</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -2929,15 +2929,15 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>163624</v>
+        <v>66656</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2945,15 +2945,15 @@
         <v>46281</v>
       </c>
       <c r="H65" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>104.97</v>
+        <v>285.74</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -2966,37 +2966,31 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>156052</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>26A0272</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>140753</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H66" t="n">
-        <v>789825</v>
+        <v>789423</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>67.54000000000001</v>
+        <v>118.12</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3009,15 +3003,15 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>136630</v>
+        <v>140718</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3025,15 +3019,15 @@
         <v>46281</v>
       </c>
       <c r="H67" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>239.16</v>
+        <v>427.44</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3046,15 +3040,15 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>163047</v>
+        <v>143381</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
@@ -3062,15 +3056,15 @@
         <v>46281</v>
       </c>
       <c r="H68" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>226.84</v>
+        <v>367.36</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3083,24 +3077,18 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>140738</v>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>0000289599</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>140709</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" s="2" t="n">
         <v>46281</v>
       </c>
@@ -3113,7 +3101,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>29.12</v>
+        <v>165.61</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3134,7 +3122,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>143384</v>
+        <v>22098</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3150,7 +3138,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>653.86</v>
+        <v>62.47</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -3171,7 +3159,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>140710</v>
+        <v>46728</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
@@ -3187,7 +3175,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>549.87</v>
+        <v>333.04</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -3208,7 +3196,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>105546</v>
+        <v>157574</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -3224,7 +3212,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>959.7</v>
+        <v>483.7</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -3245,7 +3233,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>155959</v>
+        <v>143553</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
@@ -3261,7 +3249,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>310.29</v>
+        <v>424.78</v>
       </c>
       <c r="K73" t="n">
         <v>0</v>
@@ -3282,29 +3270,23 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>12521</v>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>A44A00626</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>163624</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H74" t="n">
-        <v>31305</v>
+        <v>793186</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>LABORATORIO GLOBO LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>12.86</v>
+        <v>104.97</v>
       </c>
       <c r="K74" t="n">
         <v>0</v>
@@ -3317,31 +3299,37 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>162584</v>
-      </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
+        <v>156052</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>26A0272</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G75" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H75" t="n">
-        <v>793186</v>
+        <v>789825</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>AIRELA INDUSTRIA FARMACEUTICA LTDA</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>103.48</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
@@ -3354,15 +3342,15 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>84026</v>
+        <v>136630</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
@@ -3370,15 +3358,15 @@
         <v>46281</v>
       </c>
       <c r="H76" t="n">
-        <v>33928</v>
+        <v>30307</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>81.25</v>
+        <v>239.16</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -3391,37 +3379,31 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>123480</v>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2517347</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>163047</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H77" t="n">
-        <v>33928</v>
+        <v>30307</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>43.6</v>
+        <v>226.84</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -3442,29 +3424,29 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>79510</v>
+        <v>140738</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>0000289599</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>46844</v>
+        <v>46661</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H78" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>8.84</v>
+        <v>29.12</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -3477,37 +3459,31 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>161224</v>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>B26F1555</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>143384</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H79" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>31.97</v>
+        <v>653.86</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -3528,7 +3504,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>142053</v>
+        <v>140710</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3544,7 +3520,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>271.48</v>
+        <v>549.87</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -3565,7 +3541,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>145623</v>
+        <v>105546</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3581,7 +3557,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>208.71</v>
+        <v>959.7</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -3602,7 +3578,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>162452</v>
+        <v>155959</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3618,7 +3594,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>212.22</v>
+        <v>310.29</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -3631,31 +3607,37 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1120</v>
-      </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
+        <v>12521</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>A44A00626</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G83" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H83" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>LABORATORIO GLOBO LTDA</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>356.7</v>
+        <v>12.86</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -3668,15 +3650,15 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>142886</v>
+        <v>162584</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3684,15 +3666,15 @@
         <v>46281</v>
       </c>
       <c r="H84" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>54.88</v>
+        <v>103.48</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -3705,15 +3687,15 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>27723</v>
+        <v>84026</v>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
@@ -3721,15 +3703,15 @@
         <v>46281</v>
       </c>
       <c r="H85" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>385.19</v>
+        <v>81.25</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -3742,31 +3724,37 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>113883</v>
-      </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
+        <v>123480</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2517347</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G86" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H86" t="n">
-        <v>793186</v>
+        <v>33928</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>13.5</v>
+        <v>43.6</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -3779,31 +3767,37 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>135</v>
+        <v>72</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>158354</v>
-      </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
+        <v>79510</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>B26C2880</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G87" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H87" t="n">
-        <v>139553</v>
+        <v>47252</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>198.58</v>
+        <v>8.84</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -3824,29 +3818,29 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>95842</v>
+        <v>161224</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2519527</t>
+          <t>B26F1555</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>46753</v>
+        <v>46905</v>
       </c>
       <c r="G88" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H88" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>7.69</v>
+        <v>31.97</v>
       </c>
       <c r="K88" t="n">
         <v>0</v>
@@ -3859,37 +3853,31 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>122050</v>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>2608233</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>142053</v>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H89" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>49.61</v>
+        <v>271.48</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -3902,37 +3890,31 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>140846</v>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>2603107</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>145623</v>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H90" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>22</v>
+        <v>208.71</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -3945,37 +3927,31 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>151540</v>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>20012026</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="n">
-        <v>46569</v>
-      </c>
+        <v>162452</v>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H91" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>12.46</v>
+        <v>212.22</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3988,15 +3964,15 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>157926</v>
+        <v>1120</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
@@ -4012,7 +3988,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>22.3</v>
+        <v>356.7</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
@@ -4025,15 +4001,15 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>142054</v>
+        <v>142886</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr"/>
@@ -4049,7 +4025,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>12.8</v>
+        <v>54.88</v>
       </c>
       <c r="K93" t="n">
         <v>0</v>
@@ -4070,7 +4046,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>4006</v>
+        <v>27723</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
@@ -4086,7 +4062,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>106.69</v>
+        <v>385.19</v>
       </c>
       <c r="K94" t="n">
         <v>0</v>
@@ -4099,15 +4075,15 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>105236</v>
+        <v>113883</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
@@ -4115,15 +4091,15 @@
         <v>46281</v>
       </c>
       <c r="H95" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>1540.76</v>
+        <v>13.5</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
@@ -4136,15 +4112,15 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>145757</v>
+        <v>158354</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
@@ -4152,15 +4128,15 @@
         <v>46281</v>
       </c>
       <c r="H96" t="n">
-        <v>789423</v>
+        <v>139553</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>DINNO/PLENTY - CCM IND E COM DE PROD DESCART S/A</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>128.22</v>
+        <v>198.58</v>
       </c>
       <c r="K96" t="n">
         <v>0</v>
@@ -4173,31 +4149,37 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>105465</v>
-      </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
+        <v>95842</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2519527</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G97" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H97" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>96.3</v>
+        <v>7.69</v>
       </c>
       <c r="K97" t="n">
         <v>0</v>
@@ -4210,31 +4192,37 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>105511</v>
-      </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
+        <v>122050</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2608233</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G98" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H98" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>62.47</v>
+        <v>49.61</v>
       </c>
       <c r="K98" t="n">
         <v>0</v>
@@ -4247,31 +4235,37 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>1031</v>
-      </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
+        <v>140846</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2603107</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G99" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H99" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>256.32</v>
+        <v>22</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -4284,31 +4278,37 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>105490</v>
-      </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
+        <v>151540</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>20012026</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>46569</v>
+      </c>
       <c r="G100" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H100" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>246.9</v>
+        <v>12.46</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
@@ -4329,7 +4329,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>84530</v>
+        <v>157926</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
@@ -4337,15 +4337,15 @@
         <v>46281</v>
       </c>
       <c r="H101" t="n">
-        <v>793186</v>
+        <v>789423</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>48.14</v>
+        <v>22.3</v>
       </c>
       <c r="K101" t="n">
         <v>0</v>
@@ -4366,7 +4366,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>140516</v>
+        <v>142054</v>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
@@ -4374,15 +4374,15 @@
         <v>46281</v>
       </c>
       <c r="H102" t="n">
-        <v>30307</v>
+        <v>789423</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>108.8</v>
+        <v>12.8</v>
       </c>
       <c r="K102" t="n">
         <v>0</v>
@@ -4395,15 +4395,15 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>162989</v>
+        <v>4006</v>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
@@ -4411,15 +4411,15 @@
         <v>46281</v>
       </c>
       <c r="H103" t="n">
-        <v>796770</v>
+        <v>789423</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>155.18</v>
+        <v>106.69</v>
       </c>
       <c r="K103" t="n">
         <v>0</v>
@@ -4432,37 +4432,31 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>161944</v>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>2514837</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>105236</v>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H104" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>57.06</v>
+        <v>1540.76</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -4475,37 +4469,31 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>70696</v>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>2605007</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>145757</v>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H105" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>GEOLAB IND FARMACEUTICA S/A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>82.98</v>
+        <v>128.22</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -4518,37 +4506,31 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>154430</v>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>NEG02225</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="n">
-        <v>46692</v>
-      </c>
+        <v>105465</v>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H106" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>29.46</v>
+        <v>96.3</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -4561,15 +4543,15 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>79367</v>
+        <v>105511</v>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
@@ -4577,15 +4559,15 @@
         <v>46281</v>
       </c>
       <c r="H107" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>31.15</v>
+        <v>62.47</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -4598,15 +4580,15 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>79375</v>
+        <v>1031</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
@@ -4614,15 +4596,15 @@
         <v>46281</v>
       </c>
       <c r="H108" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>HYPERA S.A</t>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="J108" t="n">
-        <v>153.69</v>
+        <v>256.32</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -4635,24 +4617,18 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>72</v>
+        <v>142</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>140705</v>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>0000301524</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>105490</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" s="2" t="n">
         <v>46281</v>
       </c>
@@ -4665,7 +4641,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>39.98</v>
+        <v>246.9</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -4686,29 +4662,23 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>153194</v>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>0000297125</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="n">
-        <v>46508</v>
-      </c>
+        <v>84530</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H110" t="n">
-        <v>789423</v>
+        <v>793186</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>55.4</v>
+        <v>48.14</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -4729,29 +4699,23 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>143552</v>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>0000289416</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="n">
-        <v>46661</v>
-      </c>
+        <v>140516</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H111" t="n">
-        <v>789423</v>
+        <v>30307</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>CCM IND E COM DE PROD DESCARTAVEIS S/A</t>
         </is>
       </c>
       <c r="J111" t="n">
-        <v>23.94</v>
+        <v>108.8</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -4764,15 +4728,15 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>2283</v>
+        <v>162989</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -4780,15 +4744,15 @@
         <v>46281</v>
       </c>
       <c r="H112" t="n">
-        <v>789423</v>
+        <v>796770</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>FITOWAY LABORATORIO NUTRICIONAL LTDA</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>424.45</v>
+        <v>155.18</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -4801,31 +4765,37 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>141811</v>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
+        <v>161944</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2514837</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G113" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H113" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J113" t="n">
-        <v>107.64</v>
+        <v>57.06</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -4838,31 +4808,37 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>162443</v>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
+        <v>70696</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2605007</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G114" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H114" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>GEOLAB IND FARMACEUTICA S/A</t>
         </is>
       </c>
       <c r="J114" t="n">
-        <v>1546.38</v>
+        <v>82.98</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -4875,31 +4851,37 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>140716</v>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
+        <v>154430</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>NEG02225</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>46692</v>
+      </c>
       <c r="G115" s="2" t="n">
         <v>46281</v>
       </c>
       <c r="H115" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J115" t="n">
-        <v>226.5</v>
+        <v>29.46</v>
       </c>
       <c r="K115" t="n">
         <v>0</v>
@@ -4912,15 +4894,15 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>155058</v>
+        <v>79367</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -4928,15 +4910,15 @@
         <v>46281</v>
       </c>
       <c r="H116" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J116" t="n">
-        <v>1061.83</v>
+        <v>31.15</v>
       </c>
       <c r="K116" t="n">
         <v>0</v>
@@ -4949,15 +4931,15 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>145691</v>
+        <v>79375</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
@@ -4965,15 +4947,15 @@
         <v>46281</v>
       </c>
       <c r="H117" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+          <t>HYPERA S.A</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>85.43000000000001</v>
+        <v>153.69</v>
       </c>
       <c r="K117" t="n">
         <v>0</v>
@@ -4986,18 +4968,24 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>7226</v>
-      </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
+        <v>140705</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>0000301524</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G118" s="2" t="n">
         <v>46281</v>
       </c>
@@ -5010,7 +4998,7 @@
         </is>
       </c>
       <c r="J118" t="n">
-        <v>293.44</v>
+        <v>39.98</v>
       </c>
       <c r="K118" t="n">
         <v>0</v>
@@ -5023,18 +5011,24 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>105228</v>
-      </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
+        <v>153194</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>46508</v>
+      </c>
       <c r="G119" s="2" t="n">
         <v>46281</v>
       </c>
@@ -5047,7 +5041,7 @@
         </is>
       </c>
       <c r="J119" t="n">
-        <v>2753.62</v>
+        <v>55.4</v>
       </c>
       <c r="K119" t="n">
         <v>0</v>
@@ -5060,18 +5054,24 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>145423</v>
-      </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
+        <v>143552</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>0000289416</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>46661</v>
+      </c>
       <c r="G120" s="2" t="n">
         <v>46281</v>
       </c>
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>453.76</v>
+        <v>23.94</v>
       </c>
       <c r="K120" t="n">
         <v>0</v>
@@ -5105,7 +5105,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>140746</v>
+        <v>2283</v>
       </c>
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
@@ -5121,9 +5121,416 @@
         </is>
       </c>
       <c r="J121" t="n">
+        <v>424.45</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>142</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>141811</v>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H122" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>107.64</v>
+      </c>
+      <c r="K122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>142</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>162443</v>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H123" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>1546.38</v>
+      </c>
+      <c r="K123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>142</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>140716</v>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H124" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>226.5</v>
+      </c>
+      <c r="K124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>142</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>155058</v>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H125" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>1061.83</v>
+      </c>
+      <c r="K125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>142</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>145691</v>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H126" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J126" t="n">
+        <v>85.43000000000001</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>142</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>7226</v>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H127" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J127" t="n">
+        <v>293.44</v>
+      </c>
+      <c r="K127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>142</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>105228</v>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H128" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J128" t="n">
+        <v>2753.62</v>
+      </c>
+      <c r="K128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>142</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>145423</v>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H129" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>453.76</v>
+      </c>
+      <c r="K129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>142</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>140746</v>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H130" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>KLEY HERTZ DISTRIBUIDORA LTDA</t>
+        </is>
+      </c>
+      <c r="J130" t="n">
         <v>552.45</v>
       </c>
-      <c r="K121" t="n">
+      <c r="K130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>135</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>159898</v>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H131" t="n">
+        <v>789603</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>SOFTYS BRASIL LTDA</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>127.74</v>
+      </c>
+      <c r="K131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>147</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>140106</v>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H132" t="n">
+        <v>793186</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>ACCUMED PRODUTOS MEDICO HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="J132" t="n">
+        <v>1049.8</v>
+      </c>
+      <c r="K132" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:30:05
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -3398,7 +3398,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>135007</v>
+        <v>151189</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
@@ -3414,10 +3414,10 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>67.92</v>
+        <v>55</v>
       </c>
       <c r="K76" t="n">
-        <v>67.92</v>
+        <v>55</v>
       </c>
     </row>
     <row r="77">
@@ -3435,7 +3435,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>151189</v>
+        <v>151785</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
@@ -3451,10 +3451,10 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>55</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="K77" t="n">
-        <v>55</v>
+        <v>66.01000000000001</v>
       </c>
     </row>
     <row r="78">
@@ -3472,7 +3472,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>151785</v>
+        <v>135007</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>66.01000000000001</v>
+        <v>67.92</v>
       </c>
       <c r="K78" t="n">
-        <v>66.01000000000001</v>
+        <v>67.92</v>
       </c>
     </row>
     <row r="79">
@@ -5280,15 +5280,15 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>79677</v>
+        <v>19216</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>DFG8538A</t>
+          <t>B26G2054</t>
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>46692</v>
+        <v>46935</v>
       </c>
       <c r="G122" s="2" t="n">
         <v>46281</v>
@@ -5302,10 +5302,10 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>90.54000000000001</v>
+        <v>53.6</v>
       </c>
       <c r="K122" t="n">
-        <v>11.29</v>
+        <v>15.32</v>
       </c>
     </row>
     <row r="123">
@@ -5323,15 +5323,15 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>19216</v>
+        <v>79677</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>B26G2054</t>
+          <t>DFG8538A</t>
         </is>
       </c>
       <c r="F123" s="2" t="n">
-        <v>46935</v>
+        <v>46692</v>
       </c>
       <c r="G123" s="2" t="n">
         <v>46281</v>
@@ -5345,10 +5345,10 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>53.6</v>
+        <v>90.54000000000001</v>
       </c>
       <c r="K123" t="n">
-        <v>15.32</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="124">
@@ -6128,10 +6128,16 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>139483</v>
-      </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
+        <v>157169</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>0000294775</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="n">
+        <v>46753</v>
+      </c>
       <c r="G142" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6144,10 +6150,10 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>312.65</v>
+        <v>511.09</v>
       </c>
       <c r="K142" t="n">
-        <v>312.65</v>
+        <v>497.84</v>
       </c>
     </row>
     <row r="143">
@@ -6165,16 +6171,10 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>105511</v>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>0000299281</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>139483</v>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6187,10 +6187,10 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>284.39</v>
+        <v>312.65</v>
       </c>
       <c r="K143" t="n">
-        <v>284.4</v>
+        <v>312.65</v>
       </c>
     </row>
     <row r="144">
@@ -6208,16 +6208,10 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>157169</v>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>0000294775</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="n">
-        <v>46753</v>
-      </c>
+        <v>105503</v>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6230,10 +6224,10 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>511.09</v>
+        <v>66.69</v>
       </c>
       <c r="K144" t="n">
-        <v>497.84</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="145">
@@ -6251,10 +6245,16 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>105503</v>
-      </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
+        <v>105511</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>0000299281</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G145" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6267,10 +6267,10 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>66.69</v>
+        <v>284.39</v>
       </c>
       <c r="K145" t="n">
-        <v>66.7</v>
+        <v>284.4</v>
       </c>
     </row>
     <row r="146">
@@ -6331,7 +6331,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>162445</v>
+        <v>140717</v>
       </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr"/>
@@ -6347,10 +6347,10 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>61.37</v>
+        <v>217.59</v>
       </c>
       <c r="K147" t="n">
-        <v>61.37</v>
+        <v>217.59</v>
       </c>
     </row>
     <row r="148">
@@ -6368,7 +6368,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>140717</v>
+        <v>162445</v>
       </c>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr"/>
@@ -6384,10 +6384,10 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>217.59</v>
+        <v>61.37</v>
       </c>
       <c r="K148" t="n">
-        <v>217.59</v>
+        <v>61.37</v>
       </c>
     </row>
     <row r="149">
@@ -6608,10 +6608,16 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>134701</v>
-      </c>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
+        <v>159926</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>0000295698</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="n">
+        <v>46784</v>
+      </c>
       <c r="G154" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6624,10 +6630,10 @@
         </is>
       </c>
       <c r="J154" t="n">
-        <v>594.62</v>
+        <v>265.91</v>
       </c>
       <c r="K154" t="n">
-        <v>594.63</v>
+        <v>265.92</v>
       </c>
     </row>
     <row r="155">
@@ -6645,16 +6651,10 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>159926</v>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>0000295698</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="n">
-        <v>46784</v>
-      </c>
+        <v>134701</v>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
       <c r="G155" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6667,10 +6667,10 @@
         </is>
       </c>
       <c r="J155" t="n">
-        <v>265.91</v>
+        <v>594.62</v>
       </c>
       <c r="K155" t="n">
-        <v>265.92</v>
+        <v>594.63</v>
       </c>
     </row>
     <row r="156">
@@ -7174,7 +7174,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>161436</v>
+        <v>160883</v>
       </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr"/>
@@ -7190,10 +7190,10 @@
         </is>
       </c>
       <c r="J168" t="n">
-        <v>145.02</v>
+        <v>348.93</v>
       </c>
       <c r="K168" t="n">
-        <v>145.02</v>
+        <v>348.93</v>
       </c>
     </row>
     <row r="169">
@@ -7211,7 +7211,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>160883</v>
+        <v>161436</v>
       </c>
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr"/>
@@ -7227,10 +7227,10 @@
         </is>
       </c>
       <c r="J169" t="n">
-        <v>348.93</v>
+        <v>145.02</v>
       </c>
       <c r="K169" t="n">
-        <v>348.93</v>
+        <v>145.02</v>
       </c>
     </row>
     <row r="170">
@@ -11707,15 +11707,15 @@
         </is>
       </c>
       <c r="B287" t="n">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>158384</v>
+        <v>158386</v>
       </c>
       <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr"/>
@@ -11731,10 +11731,10 @@
         </is>
       </c>
       <c r="J287" t="n">
-        <v>630.17</v>
+        <v>209.97</v>
       </c>
       <c r="K287" t="n">
-        <v>630.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288">
@@ -11744,15 +11744,15 @@
         </is>
       </c>
       <c r="B288" t="n">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>158386</v>
+        <v>158384</v>
       </c>
       <c r="E288" t="inlineStr"/>
       <c r="F288" t="inlineStr"/>
@@ -11768,10 +11768,10 @@
         </is>
       </c>
       <c r="J288" t="n">
-        <v>209.97</v>
+        <v>630.17</v>
       </c>
       <c r="K288" t="n">
-        <v>0</v>
+        <v>630.16</v>
       </c>
     </row>
     <row r="289">
@@ -17441,7 +17441,7 @@
         </is>
       </c>
       <c r="D427" t="n">
-        <v>114537</v>
+        <v>149872</v>
       </c>
       <c r="E427" t="inlineStr"/>
       <c r="F427" t="inlineStr"/>
@@ -17457,10 +17457,10 @@
         </is>
       </c>
       <c r="J427" t="n">
-        <v>55.73</v>
+        <v>133.29</v>
       </c>
       <c r="K427" t="n">
-        <v>55.73</v>
+        <v>133.29</v>
       </c>
     </row>
     <row r="428">
@@ -17478,7 +17478,7 @@
         </is>
       </c>
       <c r="D428" t="n">
-        <v>151933</v>
+        <v>114537</v>
       </c>
       <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr"/>
@@ -17494,10 +17494,10 @@
         </is>
       </c>
       <c r="J428" t="n">
-        <v>130.13</v>
+        <v>55.73</v>
       </c>
       <c r="K428" t="n">
-        <v>130.13</v>
+        <v>55.73</v>
       </c>
     </row>
     <row r="429">
@@ -17515,7 +17515,7 @@
         </is>
       </c>
       <c r="D429" t="n">
-        <v>149872</v>
+        <v>151933</v>
       </c>
       <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr"/>
@@ -17531,10 +17531,10 @@
         </is>
       </c>
       <c r="J429" t="n">
-        <v>133.29</v>
+        <v>130.13</v>
       </c>
       <c r="K429" t="n">
-        <v>133.29</v>
+        <v>130.13</v>
       </c>
     </row>
     <row r="430">
@@ -20215,7 +20215,7 @@
         </is>
       </c>
       <c r="D495" t="n">
-        <v>135349</v>
+        <v>95</v>
       </c>
       <c r="E495" t="inlineStr"/>
       <c r="F495" t="inlineStr"/>
@@ -20231,10 +20231,10 @@
         </is>
       </c>
       <c r="J495" t="n">
-        <v>94.13</v>
+        <v>186.65</v>
       </c>
       <c r="K495" t="n">
-        <v>82.36</v>
+        <v>56.01</v>
       </c>
     </row>
     <row r="496">
@@ -20252,7 +20252,7 @@
         </is>
       </c>
       <c r="D496" t="n">
-        <v>95</v>
+        <v>135349</v>
       </c>
       <c r="E496" t="inlineStr"/>
       <c r="F496" t="inlineStr"/>
@@ -20268,10 +20268,10 @@
         </is>
       </c>
       <c r="J496" t="n">
-        <v>186.65</v>
+        <v>94.13</v>
       </c>
       <c r="K496" t="n">
-        <v>56.01</v>
+        <v>82.36</v>
       </c>
     </row>
     <row r="497">
@@ -20585,7 +20585,7 @@
         </is>
       </c>
       <c r="D505" t="n">
-        <v>133953</v>
+        <v>160605</v>
       </c>
       <c r="E505" t="inlineStr"/>
       <c r="F505" t="inlineStr"/>
@@ -20601,10 +20601,10 @@
         </is>
       </c>
       <c r="J505" t="n">
-        <v>226.06</v>
+        <v>146.96</v>
       </c>
       <c r="K505" t="n">
-        <v>169.54</v>
+        <v>21.01</v>
       </c>
     </row>
     <row r="506">
@@ -20622,7 +20622,7 @@
         </is>
       </c>
       <c r="D506" t="n">
-        <v>160605</v>
+        <v>133953</v>
       </c>
       <c r="E506" t="inlineStr"/>
       <c r="F506" t="inlineStr"/>
@@ -20638,10 +20638,10 @@
         </is>
       </c>
       <c r="J506" t="n">
-        <v>146.96</v>
+        <v>226.06</v>
       </c>
       <c r="K506" t="n">
-        <v>21.01</v>
+        <v>169.54</v>
       </c>
     </row>
     <row r="507">
@@ -38622,15 +38622,15 @@
         </is>
       </c>
       <c r="D962" t="n">
-        <v>7226</v>
+        <v>155058</v>
       </c>
       <c r="E962" t="inlineStr">
         <is>
-          <t>0000297214</t>
+          <t>0000281593</t>
         </is>
       </c>
       <c r="F962" s="2" t="n">
-        <v>46813</v>
+        <v>46569</v>
       </c>
       <c r="G962" s="2" t="n">
         <v>46281</v>
@@ -38644,10 +38644,10 @@
         </is>
       </c>
       <c r="J962" t="n">
-        <v>1262.69</v>
+        <v>1828.73</v>
       </c>
       <c r="K962" t="n">
-        <v>1262.7</v>
+        <v>1828.72</v>
       </c>
     </row>
     <row r="963">
@@ -38665,15 +38665,15 @@
         </is>
       </c>
       <c r="D963" t="n">
-        <v>155058</v>
+        <v>7226</v>
       </c>
       <c r="E963" t="inlineStr">
         <is>
-          <t>0000281593</t>
+          <t>0000297214</t>
         </is>
       </c>
       <c r="F963" s="2" t="n">
-        <v>46569</v>
+        <v>46813</v>
       </c>
       <c r="G963" s="2" t="n">
         <v>46281</v>
@@ -38687,10 +38687,10 @@
         </is>
       </c>
       <c r="J963" t="n">
-        <v>1828.73</v>
+        <v>1262.69</v>
       </c>
       <c r="K963" t="n">
-        <v>1828.72</v>
+        <v>1262.7</v>
       </c>
     </row>
     <row r="964">
@@ -38794,16 +38794,10 @@
         </is>
       </c>
       <c r="D966" t="n">
-        <v>142886</v>
-      </c>
-      <c r="E966" t="inlineStr">
-        <is>
-          <t>0000297310</t>
-        </is>
-      </c>
-      <c r="F966" s="2" t="n">
-        <v>46813</v>
-      </c>
+        <v>22098</v>
+      </c>
+      <c r="E966" t="inlineStr"/>
+      <c r="F966" t="inlineStr"/>
       <c r="G966" s="2" t="n">
         <v>46281</v>
       </c>
@@ -38816,10 +38810,10 @@
         </is>
       </c>
       <c r="J966" t="n">
-        <v>384.24</v>
+        <v>312.58</v>
       </c>
       <c r="K966" t="n">
-        <v>384.24</v>
+        <v>312.58</v>
       </c>
     </row>
     <row r="967">
@@ -38837,10 +38831,16 @@
         </is>
       </c>
       <c r="D967" t="n">
-        <v>22098</v>
-      </c>
-      <c r="E967" t="inlineStr"/>
-      <c r="F967" t="inlineStr"/>
+        <v>142886</v>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>0000297310</t>
+        </is>
+      </c>
+      <c r="F967" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G967" s="2" t="n">
         <v>46281</v>
       </c>
@@ -38853,10 +38853,10 @@
         </is>
       </c>
       <c r="J967" t="n">
-        <v>312.58</v>
+        <v>384.24</v>
       </c>
       <c r="K967" t="n">
-        <v>312.58</v>
+        <v>384.24</v>
       </c>
     </row>
     <row r="968">
@@ -39003,10 +39003,16 @@
         </is>
       </c>
       <c r="D971" t="n">
-        <v>105600</v>
-      </c>
-      <c r="E971" t="inlineStr"/>
-      <c r="F971" t="inlineStr"/>
+        <v>155114</v>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>0000274185</t>
+        </is>
+      </c>
+      <c r="F971" s="2" t="n">
+        <v>46478</v>
+      </c>
       <c r="G971" s="2" t="n">
         <v>46282</v>
       </c>
@@ -39019,10 +39025,10 @@
         </is>
       </c>
       <c r="J971" t="n">
-        <v>551.04</v>
+        <v>1043.5</v>
       </c>
       <c r="K971" t="n">
-        <v>551.0599999999999</v>
+        <v>820.76</v>
       </c>
     </row>
     <row r="972">
@@ -39040,16 +39046,10 @@
         </is>
       </c>
       <c r="D972" t="n">
-        <v>155114</v>
-      </c>
-      <c r="E972" t="inlineStr">
-        <is>
-          <t>0000274185</t>
-        </is>
-      </c>
-      <c r="F972" s="2" t="n">
-        <v>46478</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E972" t="inlineStr"/>
+      <c r="F972" t="inlineStr"/>
       <c r="G972" s="2" t="n">
         <v>46282</v>
       </c>
@@ -39062,10 +39062,10 @@
         </is>
       </c>
       <c r="J972" t="n">
-        <v>1043.5</v>
+        <v>551.04</v>
       </c>
       <c r="K972" t="n">
-        <v>820.76</v>
+        <v>551.0599999999999</v>
       </c>
     </row>
     <row r="973">
@@ -39163,10 +39163,16 @@
         </is>
       </c>
       <c r="D975" t="n">
-        <v>66656</v>
-      </c>
-      <c r="E975" t="inlineStr"/>
-      <c r="F975" t="inlineStr"/>
+        <v>140760</v>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>0000279041</t>
+        </is>
+      </c>
+      <c r="F975" s="2" t="n">
+        <v>46539</v>
+      </c>
       <c r="G975" s="2" t="n">
         <v>46281</v>
       </c>
@@ -39179,10 +39185,10 @@
         </is>
       </c>
       <c r="J975" t="n">
-        <v>507.56</v>
+        <v>407.68</v>
       </c>
       <c r="K975" t="n">
-        <v>507.55</v>
+        <v>407.67</v>
       </c>
     </row>
     <row r="976">
@@ -39200,16 +39206,10 @@
         </is>
       </c>
       <c r="D976" t="n">
-        <v>140760</v>
-      </c>
-      <c r="E976" t="inlineStr">
-        <is>
-          <t>0000279041</t>
-        </is>
-      </c>
-      <c r="F976" s="2" t="n">
-        <v>46539</v>
-      </c>
+        <v>66656</v>
+      </c>
+      <c r="E976" t="inlineStr"/>
+      <c r="F976" t="inlineStr"/>
       <c r="G976" s="2" t="n">
         <v>46281</v>
       </c>
@@ -39222,10 +39222,10 @@
         </is>
       </c>
       <c r="J976" t="n">
-        <v>407.68</v>
+        <v>507.56</v>
       </c>
       <c r="K976" t="n">
-        <v>407.67</v>
+        <v>507.55</v>
       </c>
     </row>
     <row r="977">
@@ -40695,7 +40695,7 @@
         </is>
       </c>
       <c r="D1013" t="n">
-        <v>141629</v>
+        <v>135185</v>
       </c>
       <c r="E1013" t="inlineStr"/>
       <c r="F1013" t="inlineStr"/>
@@ -40711,10 +40711,10 @@
         </is>
       </c>
       <c r="J1013" t="n">
-        <v>117.63</v>
+        <v>133.08</v>
       </c>
       <c r="K1013" t="n">
-        <v>35.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1014">
@@ -40732,7 +40732,7 @@
         </is>
       </c>
       <c r="D1014" t="n">
-        <v>135185</v>
+        <v>136900</v>
       </c>
       <c r="E1014" t="inlineStr"/>
       <c r="F1014" t="inlineStr"/>
@@ -40748,10 +40748,10 @@
         </is>
       </c>
       <c r="J1014" t="n">
-        <v>133.08</v>
+        <v>328.3</v>
       </c>
       <c r="K1014" t="n">
-        <v>0</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="1015">
@@ -40769,7 +40769,7 @@
         </is>
       </c>
       <c r="D1015" t="n">
-        <v>136900</v>
+        <v>141629</v>
       </c>
       <c r="E1015" t="inlineStr"/>
       <c r="F1015" t="inlineStr"/>
@@ -40785,10 +40785,10 @@
         </is>
       </c>
       <c r="J1015" t="n">
-        <v>328.3</v>
+        <v>117.63</v>
       </c>
       <c r="K1015" t="n">
-        <v>46.9</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="1016">
@@ -43112,16 +43112,10 @@
         </is>
       </c>
       <c r="D1078" t="n">
-        <v>156054</v>
-      </c>
-      <c r="E1078" t="inlineStr">
-        <is>
-          <t>26F0422</t>
-        </is>
-      </c>
-      <c r="F1078" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>156039</v>
+      </c>
+      <c r="E1078" t="inlineStr"/>
+      <c r="F1078" t="inlineStr"/>
       <c r="G1078" s="2" t="n">
         <v>46281</v>
       </c>
@@ -43134,10 +43128,10 @@
         </is>
       </c>
       <c r="J1078" t="n">
-        <v>471.93</v>
+        <v>1341.84</v>
       </c>
       <c r="K1078" t="n">
-        <v>420.74</v>
+        <v>1284.87</v>
       </c>
     </row>
     <row r="1079">
@@ -43155,10 +43149,16 @@
         </is>
       </c>
       <c r="D1079" t="n">
-        <v>156039</v>
-      </c>
-      <c r="E1079" t="inlineStr"/>
-      <c r="F1079" t="inlineStr"/>
+        <v>156054</v>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>26F0422</t>
+        </is>
+      </c>
+      <c r="F1079" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G1079" s="2" t="n">
         <v>46281</v>
       </c>
@@ -43171,10 +43171,10 @@
         </is>
       </c>
       <c r="J1079" t="n">
-        <v>1341.84</v>
+        <v>471.93</v>
       </c>
       <c r="K1079" t="n">
-        <v>1284.87</v>
+        <v>420.74</v>
       </c>
     </row>
     <row r="1080">
@@ -54808,7 +54808,7 @@
         </is>
       </c>
       <c r="D1374" t="n">
-        <v>161708</v>
+        <v>147565</v>
       </c>
       <c r="E1374" t="inlineStr"/>
       <c r="F1374" t="inlineStr"/>
@@ -54824,10 +54824,10 @@
         </is>
       </c>
       <c r="J1374" t="n">
-        <v>151.92</v>
+        <v>59.8</v>
       </c>
       <c r="K1374" t="n">
-        <v>132.93</v>
+        <v>59.8</v>
       </c>
     </row>
     <row r="1375">
@@ -54845,7 +54845,7 @@
         </is>
       </c>
       <c r="D1375" t="n">
-        <v>147565</v>
+        <v>161708</v>
       </c>
       <c r="E1375" t="inlineStr"/>
       <c r="F1375" t="inlineStr"/>
@@ -54861,10 +54861,10 @@
         </is>
       </c>
       <c r="J1375" t="n">
-        <v>59.8</v>
+        <v>151.92</v>
       </c>
       <c r="K1375" t="n">
-        <v>59.8</v>
+        <v>132.93</v>
       </c>
     </row>
     <row r="1376">
@@ -61257,7 +61257,7 @@
         </is>
       </c>
       <c r="D1535" t="n">
-        <v>135981</v>
+        <v>141485</v>
       </c>
       <c r="E1535" t="inlineStr"/>
       <c r="F1535" t="inlineStr"/>
@@ -61273,10 +61273,10 @@
         </is>
       </c>
       <c r="J1535" t="n">
-        <v>73.56</v>
+        <v>230.77</v>
       </c>
       <c r="K1535" t="n">
-        <v>55.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1536">
@@ -61294,7 +61294,7 @@
         </is>
       </c>
       <c r="D1536" t="n">
-        <v>141485</v>
+        <v>156950</v>
       </c>
       <c r="E1536" t="inlineStr"/>
       <c r="F1536" t="inlineStr"/>
@@ -61310,7 +61310,7 @@
         </is>
       </c>
       <c r="J1536" t="n">
-        <v>230.77</v>
+        <v>69</v>
       </c>
       <c r="K1536" t="n">
         <v>0</v>
@@ -61331,7 +61331,7 @@
         </is>
       </c>
       <c r="D1537" t="n">
-        <v>156950</v>
+        <v>135981</v>
       </c>
       <c r="E1537" t="inlineStr"/>
       <c r="F1537" t="inlineStr"/>
@@ -61347,10 +61347,10 @@
         </is>
       </c>
       <c r="J1537" t="n">
-        <v>69</v>
+        <v>73.56</v>
       </c>
       <c r="K1537" t="n">
-        <v>0</v>
+        <v>55.17</v>
       </c>
     </row>
     <row r="1538">
@@ -61775,7 +61775,7 @@
         </is>
       </c>
       <c r="D1549" t="n">
-        <v>135347</v>
+        <v>70</v>
       </c>
       <c r="E1549" t="inlineStr"/>
       <c r="F1549" t="inlineStr"/>
@@ -61791,10 +61791,10 @@
         </is>
       </c>
       <c r="J1549" t="n">
-        <v>47.07</v>
+        <v>63.9</v>
       </c>
       <c r="K1549" t="n">
-        <v>35.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1550">
@@ -61812,7 +61812,7 @@
         </is>
       </c>
       <c r="D1550" t="n">
-        <v>70</v>
+        <v>141068</v>
       </c>
       <c r="E1550" t="inlineStr"/>
       <c r="F1550" t="inlineStr"/>
@@ -61828,7 +61828,7 @@
         </is>
       </c>
       <c r="J1550" t="n">
-        <v>63.9</v>
+        <v>252.85</v>
       </c>
       <c r="K1550" t="n">
         <v>0</v>
@@ -61849,7 +61849,7 @@
         </is>
       </c>
       <c r="D1551" t="n">
-        <v>141068</v>
+        <v>144315</v>
       </c>
       <c r="E1551" t="inlineStr"/>
       <c r="F1551" t="inlineStr"/>
@@ -61865,7 +61865,7 @@
         </is>
       </c>
       <c r="J1551" t="n">
-        <v>252.85</v>
+        <v>144.25</v>
       </c>
       <c r="K1551" t="n">
         <v>0</v>
@@ -61886,7 +61886,7 @@
         </is>
       </c>
       <c r="D1552" t="n">
-        <v>144315</v>
+        <v>135347</v>
       </c>
       <c r="E1552" t="inlineStr"/>
       <c r="F1552" t="inlineStr"/>
@@ -61902,10 +61902,10 @@
         </is>
       </c>
       <c r="J1552" t="n">
-        <v>144.25</v>
+        <v>47.07</v>
       </c>
       <c r="K1552" t="n">
-        <v>0</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="1553">
@@ -69624,16 +69624,10 @@
         </is>
       </c>
       <c r="D1748" t="n">
-        <v>140753</v>
-      </c>
-      <c r="E1748" t="inlineStr">
-        <is>
-          <t>0000299719</t>
-        </is>
-      </c>
-      <c r="F1748" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>109681</v>
+      </c>
+      <c r="E1748" t="inlineStr"/>
+      <c r="F1748" t="inlineStr"/>
       <c r="G1748" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69646,10 +69640,10 @@
         </is>
       </c>
       <c r="J1748" t="n">
-        <v>525.25</v>
+        <v>54.1</v>
       </c>
       <c r="K1748" t="n">
-        <v>525.25</v>
+        <v>54.1</v>
       </c>
     </row>
     <row r="1749">
@@ -69667,10 +69661,16 @@
         </is>
       </c>
       <c r="D1749" t="n">
-        <v>109681</v>
-      </c>
-      <c r="E1749" t="inlineStr"/>
-      <c r="F1749" t="inlineStr"/>
+        <v>140753</v>
+      </c>
+      <c r="E1749" t="inlineStr">
+        <is>
+          <t>0000299719</t>
+        </is>
+      </c>
+      <c r="F1749" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G1749" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69683,10 +69683,10 @@
         </is>
       </c>
       <c r="J1749" t="n">
-        <v>54.1</v>
+        <v>525.25</v>
       </c>
       <c r="K1749" t="n">
-        <v>54.1</v>
+        <v>525.25</v>
       </c>
     </row>
     <row r="1750">
@@ -70024,16 +70024,10 @@
         </is>
       </c>
       <c r="D1758" t="n">
-        <v>105546</v>
-      </c>
-      <c r="E1758" t="inlineStr">
-        <is>
-          <t>0000295788</t>
-        </is>
-      </c>
-      <c r="F1758" s="2" t="n">
-        <v>46784</v>
-      </c>
+        <v>4006</v>
+      </c>
+      <c r="E1758" t="inlineStr"/>
+      <c r="F1758" t="inlineStr"/>
       <c r="G1758" s="2" t="n">
         <v>46281</v>
       </c>
@@ -70046,10 +70040,10 @@
         </is>
       </c>
       <c r="J1758" t="n">
-        <v>1672.29</v>
+        <v>926.62</v>
       </c>
       <c r="K1758" t="n">
-        <v>1672.28</v>
+        <v>926.61</v>
       </c>
     </row>
     <row r="1759">
@@ -70067,7 +70061,7 @@
         </is>
       </c>
       <c r="D1759" t="n">
-        <v>4006</v>
+        <v>145757</v>
       </c>
       <c r="E1759" t="inlineStr"/>
       <c r="F1759" t="inlineStr"/>
@@ -70083,10 +70077,10 @@
         </is>
       </c>
       <c r="J1759" t="n">
-        <v>926.62</v>
+        <v>448.76</v>
       </c>
       <c r="K1759" t="n">
-        <v>926.61</v>
+        <v>448.76</v>
       </c>
     </row>
     <row r="1760">
@@ -70104,10 +70098,16 @@
         </is>
       </c>
       <c r="D1760" t="n">
-        <v>145757</v>
-      </c>
-      <c r="E1760" t="inlineStr"/>
-      <c r="F1760" t="inlineStr"/>
+        <v>146046</v>
+      </c>
+      <c r="E1760" t="inlineStr">
+        <is>
+          <t>0000295703</t>
+        </is>
+      </c>
+      <c r="F1760" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G1760" s="2" t="n">
         <v>46281</v>
       </c>
@@ -70120,10 +70120,10 @@
         </is>
       </c>
       <c r="J1760" t="n">
-        <v>448.76</v>
+        <v>337.82</v>
       </c>
       <c r="K1760" t="n">
-        <v>448.76</v>
+        <v>337.83</v>
       </c>
     </row>
     <row r="1761">
@@ -70141,15 +70141,15 @@
         </is>
       </c>
       <c r="D1761" t="n">
-        <v>146046</v>
+        <v>105546</v>
       </c>
       <c r="E1761" t="inlineStr">
         <is>
-          <t>0000295703</t>
+          <t>0000295788</t>
         </is>
       </c>
       <c r="F1761" s="2" t="n">
-        <v>46905</v>
+        <v>46784</v>
       </c>
       <c r="G1761" s="2" t="n">
         <v>46281</v>
@@ -70163,10 +70163,10 @@
         </is>
       </c>
       <c r="J1761" t="n">
-        <v>337.82</v>
+        <v>1672.29</v>
       </c>
       <c r="K1761" t="n">
-        <v>337.83</v>
+        <v>1672.28</v>
       </c>
     </row>
     <row r="1762">
@@ -76763,7 +76763,7 @@
         </is>
       </c>
       <c r="D1933" t="n">
-        <v>151190</v>
+        <v>145580</v>
       </c>
       <c r="E1933" t="inlineStr"/>
       <c r="F1933" t="inlineStr"/>
@@ -76800,7 +76800,7 @@
         </is>
       </c>
       <c r="D1934" t="n">
-        <v>145580</v>
+        <v>151190</v>
       </c>
       <c r="E1934" t="inlineStr"/>
       <c r="F1934" t="inlineStr"/>
@@ -76985,7 +76985,7 @@
         </is>
       </c>
       <c r="D1939" t="n">
-        <v>151728</v>
+        <v>151726</v>
       </c>
       <c r="E1939" t="inlineStr"/>
       <c r="F1939" t="inlineStr"/>
@@ -77022,7 +77022,7 @@
         </is>
       </c>
       <c r="D1940" t="n">
-        <v>151726</v>
+        <v>151728</v>
       </c>
       <c r="E1940" t="inlineStr"/>
       <c r="F1940" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:15:05
</commit_message>
<xml_diff>
--- a/data/vadas.xlsx
+++ b/data/vadas.xlsx
@@ -2505,15 +2505,15 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>111732</v>
+        <v>158292</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2606032</t>
+          <t>2610693</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46874</v>
+        <v>46935</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46281</v>
@@ -2527,10 +2527,10 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>38.48</v>
+        <v>35.47</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>35.47</v>
       </c>
     </row>
     <row r="54">
@@ -2548,15 +2548,15 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>158292</v>
+        <v>111732</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2610693</t>
+          <t>2606032</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46935</v>
+        <v>46874</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46281</v>
@@ -2570,10 +2570,10 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>35.47</v>
+        <v>38.48</v>
       </c>
       <c r="K54" t="n">
-        <v>35.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -3996,10 +3996,16 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>81906</v>
-      </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
+        <v>87700</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>B26E3115</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>46905</v>
+      </c>
       <c r="G92" s="2" t="n">
         <v>46282</v>
       </c>
@@ -4012,10 +4018,10 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>811.97</v>
+        <v>524.4299999999999</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>299.69</v>
       </c>
     </row>
     <row r="93">
@@ -4033,16 +4039,10 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>87700</v>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>B26E3115</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="n">
-        <v>46905</v>
-      </c>
+        <v>81906</v>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" s="2" t="n">
         <v>46282</v>
       </c>
@@ -4055,10 +4055,10 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>524.4299999999999</v>
+        <v>811.97</v>
       </c>
       <c r="K93" t="n">
-        <v>299.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -6737,16 +6737,10 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>1600</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>0000280895</t>
-        </is>
-      </c>
-      <c r="F157" s="2" t="n">
-        <v>46539</v>
-      </c>
+        <v>161436</v>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
       <c r="G157" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6759,10 +6753,10 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>156.78</v>
+        <v>145.02</v>
       </c>
       <c r="K157" t="n">
-        <v>156.78</v>
+        <v>145.02</v>
       </c>
     </row>
     <row r="158">
@@ -6780,10 +6774,16 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>161436</v>
-      </c>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
+        <v>1600</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>0000280895</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="n">
+        <v>46539</v>
+      </c>
       <c r="G158" s="2" t="n">
         <v>46281</v>
       </c>
@@ -6796,10 +6796,10 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>145.02</v>
+        <v>156.78</v>
       </c>
       <c r="K158" t="n">
-        <v>145.02</v>
+        <v>156.78</v>
       </c>
     </row>
     <row r="159">
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>155228</v>
+        <v>153650</v>
       </c>
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr"/>
@@ -10548,10 +10548,10 @@
         </is>
       </c>
       <c r="J256" t="n">
-        <v>212.33</v>
+        <v>1079.91</v>
       </c>
       <c r="K256" t="n">
-        <v>174.86</v>
+        <v>839.9299999999999</v>
       </c>
     </row>
     <row r="257">
@@ -10569,7 +10569,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>153650</v>
+        <v>155228</v>
       </c>
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr"/>
@@ -10585,10 +10585,10 @@
         </is>
       </c>
       <c r="J257" t="n">
-        <v>1079.91</v>
+        <v>212.33</v>
       </c>
       <c r="K257" t="n">
-        <v>839.9299999999999</v>
+        <v>174.86</v>
       </c>
     </row>
     <row r="258">
@@ -13455,15 +13455,15 @@
         </is>
       </c>
       <c r="B331" t="n">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>159404</v>
+        <v>135013</v>
       </c>
       <c r="E331" t="inlineStr"/>
       <c r="F331" t="inlineStr"/>
@@ -13479,10 +13479,10 @@
         </is>
       </c>
       <c r="J331" t="n">
-        <v>157.37</v>
+        <v>1820.86</v>
       </c>
       <c r="K331" t="n">
-        <v>31.49</v>
+        <v>1820.85</v>
       </c>
     </row>
     <row r="332">
@@ -13492,15 +13492,15 @@
         </is>
       </c>
       <c r="B332" t="n">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>135013</v>
+        <v>151729</v>
       </c>
       <c r="E332" t="inlineStr"/>
       <c r="F332" t="inlineStr"/>
@@ -13516,10 +13516,10 @@
         </is>
       </c>
       <c r="J332" t="n">
-        <v>1820.86</v>
+        <v>20.34</v>
       </c>
       <c r="K332" t="n">
-        <v>1820.85</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="333">
@@ -13537,7 +13537,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>151729</v>
+        <v>159404</v>
       </c>
       <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr"/>
@@ -13553,10 +13553,10 @@
         </is>
       </c>
       <c r="J333" t="n">
-        <v>20.34</v>
+        <v>157.37</v>
       </c>
       <c r="K333" t="n">
-        <v>20.34</v>
+        <v>31.49</v>
       </c>
     </row>
     <row r="334">
@@ -24437,15 +24437,15 @@
         </is>
       </c>
       <c r="D607" t="n">
-        <v>111694</v>
+        <v>105180</v>
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>2606425</t>
+          <t>2609021</t>
         </is>
       </c>
       <c r="F607" s="2" t="n">
-        <v>46874</v>
+        <v>46935</v>
       </c>
       <c r="G607" s="2" t="n">
         <v>46281</v>
@@ -24459,7 +24459,7 @@
         </is>
       </c>
       <c r="J607" t="n">
-        <v>20.39</v>
+        <v>37.02</v>
       </c>
       <c r="K607" t="n">
         <v>0</v>
@@ -24480,15 +24480,15 @@
         </is>
       </c>
       <c r="D608" t="n">
-        <v>105180</v>
+        <v>111694</v>
       </c>
       <c r="E608" t="inlineStr">
         <is>
-          <t>2609021</t>
+          <t>2606425</t>
         </is>
       </c>
       <c r="F608" s="2" t="n">
-        <v>46935</v>
+        <v>46874</v>
       </c>
       <c r="G608" s="2" t="n">
         <v>46281</v>
@@ -24502,7 +24502,7 @@
         </is>
       </c>
       <c r="J608" t="n">
-        <v>37.02</v>
+        <v>20.39</v>
       </c>
       <c r="K608" t="n">
         <v>0</v>
@@ -25618,7 +25618,7 @@
         </is>
       </c>
       <c r="D636" t="n">
-        <v>143798</v>
+        <v>134223</v>
       </c>
       <c r="E636" t="inlineStr"/>
       <c r="F636" t="inlineStr"/>
@@ -25634,10 +25634,10 @@
         </is>
       </c>
       <c r="J636" t="n">
-        <v>22.15</v>
+        <v>149.7</v>
       </c>
       <c r="K636" t="n">
-        <v>22.15</v>
+        <v>149.7</v>
       </c>
     </row>
     <row r="637">
@@ -25655,7 +25655,7 @@
         </is>
       </c>
       <c r="D637" t="n">
-        <v>134223</v>
+        <v>143798</v>
       </c>
       <c r="E637" t="inlineStr"/>
       <c r="F637" t="inlineStr"/>
@@ -25671,10 +25671,10 @@
         </is>
       </c>
       <c r="J637" t="n">
-        <v>149.7</v>
+        <v>22.15</v>
       </c>
       <c r="K637" t="n">
-        <v>149.7</v>
+        <v>22.15</v>
       </c>
     </row>
     <row r="638">
@@ -28810,10 +28810,16 @@
         </is>
       </c>
       <c r="D714" t="n">
-        <v>105600</v>
-      </c>
-      <c r="E714" t="inlineStr"/>
-      <c r="F714" t="inlineStr"/>
+        <v>140747</v>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>0000297182</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="n">
+        <v>46813</v>
+      </c>
       <c r="G714" s="2" t="n">
         <v>46281</v>
       </c>
@@ -28826,10 +28832,10 @@
         </is>
       </c>
       <c r="J714" t="n">
-        <v>849.13</v>
+        <v>706.24</v>
       </c>
       <c r="K714" t="n">
-        <v>849.12</v>
+        <v>706.24</v>
       </c>
     </row>
     <row r="715">
@@ -28847,16 +28853,10 @@
         </is>
       </c>
       <c r="D715" t="n">
-        <v>115223</v>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>0000287656</t>
-        </is>
-      </c>
-      <c r="F715" s="2" t="n">
-        <v>46631</v>
-      </c>
+        <v>105600</v>
+      </c>
+      <c r="E715" t="inlineStr"/>
+      <c r="F715" t="inlineStr"/>
       <c r="G715" s="2" t="n">
         <v>46281</v>
       </c>
@@ -28869,10 +28869,10 @@
         </is>
       </c>
       <c r="J715" t="n">
-        <v>59.61</v>
+        <v>849.13</v>
       </c>
       <c r="K715" t="n">
-        <v>59.61</v>
+        <v>849.12</v>
       </c>
     </row>
     <row r="716">
@@ -28890,15 +28890,15 @@
         </is>
       </c>
       <c r="D716" t="n">
-        <v>140747</v>
+        <v>115223</v>
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>0000297182</t>
+          <t>0000287656</t>
         </is>
       </c>
       <c r="F716" s="2" t="n">
-        <v>46813</v>
+        <v>46631</v>
       </c>
       <c r="G716" s="2" t="n">
         <v>46281</v>
@@ -28912,10 +28912,10 @@
         </is>
       </c>
       <c r="J716" t="n">
-        <v>706.24</v>
+        <v>59.61</v>
       </c>
       <c r="K716" t="n">
-        <v>706.24</v>
+        <v>59.61</v>
       </c>
     </row>
     <row r="717">
@@ -38659,10 +38659,16 @@
         </is>
       </c>
       <c r="D963" t="n">
-        <v>141180</v>
-      </c>
-      <c r="E963" t="inlineStr"/>
-      <c r="F963" t="inlineStr"/>
+        <v>153194</v>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>0000297125</t>
+        </is>
+      </c>
+      <c r="F963" s="2" t="n">
+        <v>46508</v>
+      </c>
       <c r="G963" s="2" t="n">
         <v>46281</v>
       </c>
@@ -38675,10 +38681,10 @@
         </is>
       </c>
       <c r="J963" t="n">
-        <v>403.06</v>
+        <v>2073.07</v>
       </c>
       <c r="K963" t="n">
-        <v>403.06</v>
+        <v>2179.35</v>
       </c>
     </row>
     <row r="964">
@@ -38696,16 +38702,10 @@
         </is>
       </c>
       <c r="D964" t="n">
-        <v>153194</v>
-      </c>
-      <c r="E964" t="inlineStr">
-        <is>
-          <t>0000297125</t>
-        </is>
-      </c>
-      <c r="F964" s="2" t="n">
-        <v>46508</v>
-      </c>
+        <v>141180</v>
+      </c>
+      <c r="E964" t="inlineStr"/>
+      <c r="F964" t="inlineStr"/>
       <c r="G964" s="2" t="n">
         <v>46281</v>
       </c>
@@ -38718,10 +38718,10 @@
         </is>
       </c>
       <c r="J964" t="n">
-        <v>2073.07</v>
+        <v>403.06</v>
       </c>
       <c r="K964" t="n">
-        <v>2179.35</v>
+        <v>403.06</v>
       </c>
     </row>
     <row r="965">
@@ -39426,19 +39426,19 @@
         </is>
       </c>
       <c r="B982" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C982" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D982" t="n">
-        <v>140747</v>
+        <v>7226</v>
       </c>
       <c r="E982" t="inlineStr">
         <is>
-          <t>0000297182</t>
+          <t>0000297214</t>
         </is>
       </c>
       <c r="F982" s="2" t="n">
@@ -39456,10 +39456,10 @@
         </is>
       </c>
       <c r="J982" t="n">
-        <v>53.25</v>
+        <v>1262.69</v>
       </c>
       <c r="K982" t="n">
-        <v>53.25</v>
+        <v>1262.7</v>
       </c>
     </row>
     <row r="983">
@@ -39469,19 +39469,19 @@
         </is>
       </c>
       <c r="B983" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C983" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D983" t="n">
-        <v>7226</v>
+        <v>140747</v>
       </c>
       <c r="E983" t="inlineStr">
         <is>
-          <t>0000297214</t>
+          <t>0000297182</t>
         </is>
       </c>
       <c r="F983" s="2" t="n">
@@ -39499,10 +39499,10 @@
         </is>
       </c>
       <c r="J983" t="n">
-        <v>1262.69</v>
+        <v>53.25</v>
       </c>
       <c r="K983" t="n">
-        <v>1262.7</v>
+        <v>53.25</v>
       </c>
     </row>
     <row r="984">
@@ -39758,23 +39758,23 @@
         </is>
       </c>
       <c r="B990" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C990" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D990" t="n">
-        <v>143658</v>
+        <v>162452</v>
       </c>
       <c r="E990" t="inlineStr">
         <is>
-          <t>0000289887</t>
+          <t>0000297547</t>
         </is>
       </c>
       <c r="F990" s="2" t="n">
-        <v>46661</v>
+        <v>46813</v>
       </c>
       <c r="G990" s="2" t="n">
         <v>46281</v>
@@ -39788,10 +39788,10 @@
         </is>
       </c>
       <c r="J990" t="n">
-        <v>72.78</v>
+        <v>212.24</v>
       </c>
       <c r="K990" t="n">
-        <v>72.78</v>
+        <v>212.23</v>
       </c>
     </row>
     <row r="991">
@@ -39801,23 +39801,23 @@
         </is>
       </c>
       <c r="B991" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C991" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D991" t="n">
-        <v>162452</v>
+        <v>143658</v>
       </c>
       <c r="E991" t="inlineStr">
         <is>
-          <t>0000297547</t>
+          <t>0000289887</t>
         </is>
       </c>
       <c r="F991" s="2" t="n">
-        <v>46813</v>
+        <v>46661</v>
       </c>
       <c r="G991" s="2" t="n">
         <v>46281</v>
@@ -39831,10 +39831,10 @@
         </is>
       </c>
       <c r="J991" t="n">
-        <v>212.24</v>
+        <v>72.78</v>
       </c>
       <c r="K991" t="n">
-        <v>212.23</v>
+        <v>72.78</v>
       </c>
     </row>
     <row r="992">
@@ -41768,7 +41768,7 @@
         </is>
       </c>
       <c r="D1042" t="n">
-        <v>162638</v>
+        <v>162704</v>
       </c>
       <c r="E1042" t="inlineStr"/>
       <c r="F1042" t="inlineStr"/>
@@ -41784,10 +41784,10 @@
         </is>
       </c>
       <c r="J1042" t="n">
-        <v>61.21</v>
+        <v>126.09</v>
       </c>
       <c r="K1042" t="n">
-        <v>61.21</v>
+        <v>126.09</v>
       </c>
     </row>
     <row r="1043">
@@ -41805,7 +41805,7 @@
         </is>
       </c>
       <c r="D1043" t="n">
-        <v>162704</v>
+        <v>162638</v>
       </c>
       <c r="E1043" t="inlineStr"/>
       <c r="F1043" t="inlineStr"/>
@@ -41821,10 +41821,10 @@
         </is>
       </c>
       <c r="J1043" t="n">
-        <v>126.09</v>
+        <v>61.21</v>
       </c>
       <c r="K1043" t="n">
-        <v>126.09</v>
+        <v>61.21</v>
       </c>
     </row>
     <row r="1044">
@@ -42064,7 +42064,7 @@
         </is>
       </c>
       <c r="D1050" t="n">
-        <v>156656</v>
+        <v>151445</v>
       </c>
       <c r="E1050" t="inlineStr"/>
       <c r="F1050" t="inlineStr"/>
@@ -42080,10 +42080,10 @@
         </is>
       </c>
       <c r="J1050" t="n">
-        <v>2456.87</v>
+        <v>4725</v>
       </c>
       <c r="K1050" t="n">
-        <v>2078.88</v>
+        <v>4173.02</v>
       </c>
     </row>
     <row r="1051">
@@ -42101,7 +42101,7 @@
         </is>
       </c>
       <c r="D1051" t="n">
-        <v>151445</v>
+        <v>156656</v>
       </c>
       <c r="E1051" t="inlineStr"/>
       <c r="F1051" t="inlineStr"/>
@@ -42117,10 +42117,10 @@
         </is>
       </c>
       <c r="J1051" t="n">
-        <v>4725</v>
+        <v>2456.87</v>
       </c>
       <c r="K1051" t="n">
-        <v>4173.02</v>
+        <v>2078.88</v>
       </c>
     </row>
     <row r="1052">
@@ -47557,7 +47557,7 @@
         </is>
       </c>
       <c r="D1191" t="n">
-        <v>145579</v>
+        <v>145583</v>
       </c>
       <c r="E1191" t="inlineStr"/>
       <c r="F1191" t="inlineStr"/>
@@ -47594,7 +47594,7 @@
         </is>
       </c>
       <c r="D1192" t="n">
-        <v>145583</v>
+        <v>145579</v>
       </c>
       <c r="E1192" t="inlineStr"/>
       <c r="F1192" t="inlineStr"/>
@@ -51786,18 +51786,24 @@
         </is>
       </c>
       <c r="B1294" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C1294" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D1294" t="n">
-        <v>10359</v>
-      </c>
-      <c r="E1294" t="inlineStr"/>
-      <c r="F1294" t="inlineStr"/>
+        <v>155062</v>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>0000295009</t>
+        </is>
+      </c>
+      <c r="F1294" s="2" t="n">
+        <v>47150</v>
+      </c>
       <c r="G1294" s="2" t="n">
         <v>46281</v>
       </c>
@@ -51810,10 +51816,10 @@
         </is>
       </c>
       <c r="J1294" t="n">
-        <v>50.03</v>
+        <v>2311.09</v>
       </c>
       <c r="K1294" t="n">
-        <v>50.03</v>
+        <v>2311.09</v>
       </c>
     </row>
     <row r="1295">
@@ -51823,24 +51829,18 @@
         </is>
       </c>
       <c r="B1295" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C1295" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D1295" t="n">
-        <v>155062</v>
-      </c>
-      <c r="E1295" t="inlineStr">
-        <is>
-          <t>0000295009</t>
-        </is>
-      </c>
-      <c r="F1295" s="2" t="n">
-        <v>47150</v>
-      </c>
+        <v>10359</v>
+      </c>
+      <c r="E1295" t="inlineStr"/>
+      <c r="F1295" t="inlineStr"/>
       <c r="G1295" s="2" t="n">
         <v>46281</v>
       </c>
@@ -51853,10 +51853,10 @@
         </is>
       </c>
       <c r="J1295" t="n">
-        <v>2311.09</v>
+        <v>50.03</v>
       </c>
       <c r="K1295" t="n">
-        <v>2311.09</v>
+        <v>50.03</v>
       </c>
     </row>
     <row r="1296">
@@ -53032,7 +53032,7 @@
         </is>
       </c>
       <c r="D1326" t="n">
-        <v>145834</v>
+        <v>145835</v>
       </c>
       <c r="E1326" t="inlineStr"/>
       <c r="F1326" t="inlineStr"/>
@@ -53069,7 +53069,7 @@
         </is>
       </c>
       <c r="D1327" t="n">
-        <v>145835</v>
+        <v>145834</v>
       </c>
       <c r="E1327" t="inlineStr"/>
       <c r="F1327" t="inlineStr"/>
@@ -59738,15 +59738,15 @@
         </is>
       </c>
       <c r="D1498" t="n">
-        <v>79510</v>
+        <v>161224</v>
       </c>
       <c r="E1498" t="inlineStr">
         <is>
-          <t>B26C2880</t>
+          <t>B26F1555</t>
         </is>
       </c>
       <c r="F1498" s="2" t="n">
-        <v>46844</v>
+        <v>46905</v>
       </c>
       <c r="G1498" s="2" t="n">
         <v>46281</v>
@@ -59760,7 +59760,7 @@
         </is>
       </c>
       <c r="J1498" t="n">
-        <v>8.84</v>
+        <v>31.97</v>
       </c>
       <c r="K1498" t="n">
         <v>0</v>
@@ -59781,15 +59781,15 @@
         </is>
       </c>
       <c r="D1499" t="n">
-        <v>161224</v>
+        <v>79510</v>
       </c>
       <c r="E1499" t="inlineStr">
         <is>
-          <t>B26F1555</t>
+          <t>B26C2880</t>
         </is>
       </c>
       <c r="F1499" s="2" t="n">
-        <v>46905</v>
+        <v>46844</v>
       </c>
       <c r="G1499" s="2" t="n">
         <v>46281</v>
@@ -59803,7 +59803,7 @@
         </is>
       </c>
       <c r="J1499" t="n">
-        <v>31.97</v>
+        <v>8.84</v>
       </c>
       <c r="K1499" t="n">
         <v>0</v>
@@ -60763,23 +60763,23 @@
         </is>
       </c>
       <c r="B1523" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C1523" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D1523" t="n">
-        <v>144646</v>
+        <v>143551</v>
       </c>
       <c r="E1523" t="inlineStr">
         <is>
-          <t>30472</t>
+          <t>0000292120</t>
         </is>
       </c>
       <c r="F1523" s="2" t="n">
-        <v>46753</v>
+        <v>46722</v>
       </c>
       <c r="G1523" s="2" t="n">
         <v>46281</v>
@@ -60793,10 +60793,10 @@
         </is>
       </c>
       <c r="J1523" t="n">
-        <v>60.51</v>
+        <v>106.92</v>
       </c>
       <c r="K1523" t="n">
-        <v>60.51</v>
+        <v>106.92</v>
       </c>
     </row>
     <row r="1524">
@@ -60806,23 +60806,23 @@
         </is>
       </c>
       <c r="B1524" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C1524" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D1524" t="n">
-        <v>143551</v>
+        <v>144646</v>
       </c>
       <c r="E1524" t="inlineStr">
         <is>
-          <t>0000292120</t>
+          <t>30472</t>
         </is>
       </c>
       <c r="F1524" s="2" t="n">
-        <v>46722</v>
+        <v>46753</v>
       </c>
       <c r="G1524" s="2" t="n">
         <v>46281</v>
@@ -60836,10 +60836,10 @@
         </is>
       </c>
       <c r="J1524" t="n">
-        <v>106.92</v>
+        <v>60.51</v>
       </c>
       <c r="K1524" t="n">
-        <v>106.92</v>
+        <v>60.51</v>
       </c>
     </row>
     <row r="1525">
@@ -62803,15 +62803,15 @@
         </is>
       </c>
       <c r="B1577" t="n">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C1577" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="D1577" t="n">
-        <v>159127</v>
+        <v>1732</v>
       </c>
       <c r="E1577" t="inlineStr"/>
       <c r="F1577" t="inlineStr"/>
@@ -62827,10 +62827,10 @@
         </is>
       </c>
       <c r="J1577" t="n">
-        <v>3967.89</v>
+        <v>729.36</v>
       </c>
       <c r="K1577" t="n">
-        <v>379.78</v>
+        <v>639.51</v>
       </c>
     </row>
     <row r="1578">
@@ -62840,15 +62840,15 @@
         </is>
       </c>
       <c r="B1578" t="n">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C1578" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D1578" t="n">
-        <v>1732</v>
+        <v>159127</v>
       </c>
       <c r="E1578" t="inlineStr"/>
       <c r="F1578" t="inlineStr"/>
@@ -62864,10 +62864,10 @@
         </is>
       </c>
       <c r="J1578" t="n">
-        <v>729.36</v>
+        <v>3967.89</v>
       </c>
       <c r="K1578" t="n">
-        <v>639.51</v>
+        <v>379.78</v>
       </c>
     </row>
     <row r="1579">
@@ -69815,10 +69815,16 @@
         </is>
       </c>
       <c r="D1753" t="n">
-        <v>145757</v>
-      </c>
-      <c r="E1753" t="inlineStr"/>
-      <c r="F1753" t="inlineStr"/>
+        <v>140753</v>
+      </c>
+      <c r="E1753" t="inlineStr">
+        <is>
+          <t>0000299719</t>
+        </is>
+      </c>
+      <c r="F1753" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G1753" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69831,10 +69837,10 @@
         </is>
       </c>
       <c r="J1753" t="n">
-        <v>448.76</v>
+        <v>525.25</v>
       </c>
       <c r="K1753" t="n">
-        <v>448.76</v>
+        <v>525.25</v>
       </c>
     </row>
     <row r="1754">
@@ -69844,18 +69850,24 @@
         </is>
       </c>
       <c r="B1754" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C1754" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D1754" t="n">
-        <v>140716</v>
-      </c>
-      <c r="E1754" t="inlineStr"/>
-      <c r="F1754" t="inlineStr"/>
+        <v>162453</v>
+      </c>
+      <c r="E1754" t="inlineStr">
+        <is>
+          <t>0000301177</t>
+        </is>
+      </c>
+      <c r="F1754" s="2" t="n">
+        <v>46844</v>
+      </c>
       <c r="G1754" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69868,10 +69880,10 @@
         </is>
       </c>
       <c r="J1754" t="n">
-        <v>33.98</v>
+        <v>151.35</v>
       </c>
       <c r="K1754" t="n">
-        <v>33.98</v>
+        <v>151.35</v>
       </c>
     </row>
     <row r="1755">
@@ -69889,16 +69901,10 @@
         </is>
       </c>
       <c r="D1755" t="n">
-        <v>140753</v>
-      </c>
-      <c r="E1755" t="inlineStr">
-        <is>
-          <t>0000299719</t>
-        </is>
-      </c>
-      <c r="F1755" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>145757</v>
+      </c>
+      <c r="E1755" t="inlineStr"/>
+      <c r="F1755" t="inlineStr"/>
       <c r="G1755" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69911,10 +69917,10 @@
         </is>
       </c>
       <c r="J1755" t="n">
-        <v>525.25</v>
+        <v>448.76</v>
       </c>
       <c r="K1755" t="n">
-        <v>525.25</v>
+        <v>448.76</v>
       </c>
     </row>
     <row r="1756">
@@ -69924,24 +69930,18 @@
         </is>
       </c>
       <c r="B1756" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C1756" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D1756" t="n">
-        <v>162453</v>
-      </c>
-      <c r="E1756" t="inlineStr">
-        <is>
-          <t>0000301177</t>
-        </is>
-      </c>
-      <c r="F1756" s="2" t="n">
-        <v>46844</v>
-      </c>
+        <v>140716</v>
+      </c>
+      <c r="E1756" t="inlineStr"/>
+      <c r="F1756" t="inlineStr"/>
       <c r="G1756" s="2" t="n">
         <v>46281</v>
       </c>
@@ -69954,10 +69954,10 @@
         </is>
       </c>
       <c r="J1756" t="n">
-        <v>151.35</v>
+        <v>33.98</v>
       </c>
       <c r="K1756" t="n">
-        <v>151.35</v>
+        <v>33.98</v>
       </c>
     </row>
     <row r="1757">
@@ -70172,7 +70172,7 @@
         </is>
       </c>
       <c r="D1762" t="n">
-        <v>159382</v>
+        <v>105236</v>
       </c>
       <c r="E1762" t="inlineStr"/>
       <c r="F1762" t="inlineStr"/>
@@ -70188,10 +70188,10 @@
         </is>
       </c>
       <c r="J1762" t="n">
-        <v>163.63</v>
+        <v>2592.72</v>
       </c>
       <c r="K1762" t="n">
-        <v>163.63</v>
+        <v>2548.99</v>
       </c>
     </row>
     <row r="1763">
@@ -70209,7 +70209,7 @@
         </is>
       </c>
       <c r="D1763" t="n">
-        <v>105236</v>
+        <v>159382</v>
       </c>
       <c r="E1763" t="inlineStr"/>
       <c r="F1763" t="inlineStr"/>
@@ -70225,10 +70225,10 @@
         </is>
       </c>
       <c r="J1763" t="n">
-        <v>2592.72</v>
+        <v>163.63</v>
       </c>
       <c r="K1763" t="n">
-        <v>2548.99</v>
+        <v>163.63</v>
       </c>
     </row>
     <row r="1764">
@@ -74609,7 +74609,7 @@
         </is>
       </c>
       <c r="D1879" t="n">
-        <v>156161</v>
+        <v>153947</v>
       </c>
       <c r="E1879" t="inlineStr"/>
       <c r="F1879" t="inlineStr"/>
@@ -74625,10 +74625,10 @@
         </is>
       </c>
       <c r="J1879" t="n">
-        <v>801.86</v>
+        <v>3359.67</v>
       </c>
       <c r="K1879" t="n">
-        <v>534.47</v>
+        <v>2971.93</v>
       </c>
     </row>
     <row r="1880">
@@ -74646,7 +74646,7 @@
         </is>
       </c>
       <c r="D1880" t="n">
-        <v>153947</v>
+        <v>156161</v>
       </c>
       <c r="E1880" t="inlineStr"/>
       <c r="F1880" t="inlineStr"/>
@@ -74662,10 +74662,10 @@
         </is>
       </c>
       <c r="J1880" t="n">
-        <v>3359.67</v>
+        <v>801.86</v>
       </c>
       <c r="K1880" t="n">
-        <v>2971.93</v>
+        <v>534.47</v>
       </c>
     </row>
     <row r="1881">

</xml_diff>